<commit_message>
feat: update official photos for Rahul, Majin, Ravneet, Jason and clear photos for Chris Donovan and Ein
</commit_message>
<xml_diff>
--- a/exports/Cayman_Super_Kings_Complete_Database.xlsx
+++ b/exports/Cayman_Super_Kings_Complete_Database.xlsx
@@ -1609,12 +1609,12 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>assets/players/real/Chris.jpg</t>
+          <t/>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1701,12 +1701,12 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>assets/players/real/Ein-Majin-solo.jpg</t>
+          <t/>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: remove news section and navbar link, update Muthukumar official photo, remove all Drive links and HUD cutouts from squad cards
</commit_message>
<xml_diff>
--- a/exports/Cayman_Super_Kings_Complete_Database.xlsx
+++ b/exports/Cayman_Super_Kings_Complete_Database.xlsx
@@ -418,7 +418,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1xdI7M2cpiq5qK1VQx252zj5MWqQJ7eHR/view?usp=drivesdk</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -510,7 +510,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -602,7 +602,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -786,7 +786,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -965,12 +965,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>assets/players/real/dfc6af5a-1c01-458c-8b44-26fce836510d.jpg</t>
+          <t>assets/players/real/Muthukumar-Rajenderan.jpg</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1890,7 +1890,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>https://drive.google.com/drive/folders/1rYNaOJZCnTV7RrFFjOI08XvzURHpywHH</t>
+          <t/>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: real CICA CricClubs match data with dynamic API sync, futuristic HUD animations, and full responsiveness
</commit_message>
<xml_diff>
--- a/exports/Cayman_Super_Kings_Complete_Database.xlsx
+++ b/exports/Cayman_Super_Kings_Complete_Database.xlsx
@@ -2098,12 +2098,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>csk-vs-tigers-super-league-t20-2026</t>
+          <t>csk-vs-tamilnadu-daniel-morris-t20-final</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League T20</t>
+          <t>Daniel Morris Division 2 T20 Championship</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2113,17 +2113,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>George Town Tigers</t>
+          <t>Tamilnadu Cricket Club</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>GTT</t>
+          <t>TNCC</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2025-04-06</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>178/4</t>
+          <t>174/5</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>142/9</t>
+          <t>156/8</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 36 runs</t>
+          <t>Cayman Super Kings won by 18 runs</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -2173,12 +2173,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Rahul Garg (68* &amp; 2/19)</t>
+          <t>Rahul Garg (64 off 41 &amp; 2/18)</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>A commanding all-round performance led by skipper Rahul Garg guided the Super Kings to an emphatic 36-run victory over rivals George Town Tigers in front of an electric crowd at Jimmy Powell Oval.</t>
+          <t>In an electric Daniel Morris Division 2 T20 Finals clash, skipper Rahul Garg anchored a high-stakes 174 total before a lethal bowling spell sealed an 18-run championship victory for CSK at Jimmy Powell Oval.</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -2195,72 +2195,72 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>csk-vs-seven-mile-strikers-super-league-40over</t>
+          <t>csk-vs-village-greenies-super-league-t20-2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League 40 Over</t>
+          <t>Cayman Cricket Super League T20</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>40-Over</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Seven Mile Strikers</t>
+          <t>Village Greenies</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>VGC</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Smith Road Oval, George Town</t>
+          <t>Jimmy Powell Oval, George Town</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2025-05-18</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>248/7</t>
+          <t>182/4</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>212/10</t>
+          <t>165/7</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>37.4</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 36 runs</t>
+          <t>Cayman Super Kings won by 17 runs</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -2270,12 +2270,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Christopher Balraj (104 off 92 balls)</t>
+          <t>Christopher Balraj (78 off 46)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Christopher Balraj posted a sublime 104 to anchor a daunting 248 total before Sahil Singh ripped through the Strikers top order with 4/38.</t>
+          <t>Opening batter Christopher Balraj unleashed an explosive 78 to propel CSK to 182, followed by a clinical 3-wicket defense from Sahil Singh against the Greenies.</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -2292,72 +2292,72 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>csk-vs-greenies-elite-50-over-2026</t>
+          <t>csk-vs-west-bay-warriors-super-league-t20-2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cayman Cricket Elite 50 Over League</t>
+          <t>Cayman Cricket Super League T20</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>50-Over</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Village Greenies</t>
+          <t>West Bay Warriors</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>VGC</t>
+          <t>WBW</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Jimmy Powell Oval, George Town</t>
+          <t>Smith Road Oval, George Town</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2025-06-08</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>284/6</t>
+          <t>168/6</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>241/10</t>
+          <t>164/8</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>46.2</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 43 runs</t>
+          <t>Cayman Super Kings won by 4 wickets</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -2367,12 +2367,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Gokul Krishnan (86 off 78)</t>
+          <t>Gokul Krishnan (52* off 31)</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Gokul Krishnan and Rahul Garg forged a crucial 140-run partnership in the 50-over fixture before Ravneet Verma claimed 4 wickets to secure victory.</t>
+          <t>Wicketkeeper batsman Gokul Krishnan struck three consecutive boundaries in the penultimate over to chase down 165 against West Bay Warriors.</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -2389,32 +2389,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>csk-vs-bodden-town-elite-t20-2026</t>
+          <t>csk-vs-seven-mile-strikers-super-league-40over-2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Cayman Cricket Elite T20 League</t>
+          <t>Cayman Cricket Super League 40 Over</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>40-Over</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Bodden Town CC</t>
+          <t>Seven Mile Strikers</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>BTCC</t>
+          <t>SMS</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -2424,37 +2424,37 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2025-07-13</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>164/5</t>
+          <t>256/7</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>19.2</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>163/8</t>
+          <t>221/10</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>38.2</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 5 wickets</t>
+          <t>Cayman Super Kings won by 35 runs</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Gokul Krishnan (48* off 26)</t>
+          <t>Muthukumar Rajenderan (4/36)</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Chasing 164, wicketkeeper Gokul Krishnan kept his cool with a boundary blitz in the penultimate over to secure two vital points.</t>
+          <t>A disciplined bowling assault from Muthukumar Rajenderan (4/36) dismantled Seven Mile Strikers chasing 257 in the 40-over championship fixture.</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -2486,32 +2486,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>csk-vs-north-side-super-league-t20-2026</t>
+          <t>csk-vs-police-cc-super-league-40over-2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League T20</t>
+          <t>Cayman Cricket Super League 40 Over</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>40-Over</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>North Side XI</t>
+          <t>Police Cricket Club</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>NSXI</t>
+          <t>PCC</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2521,37 +2521,37 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2025-08-10</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>185/3</t>
+          <t>238/8</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>151/8</t>
+          <t>210/10</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>37.5</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 34 runs</t>
+          <t>Cayman Super Kings won by 28 runs</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -2561,12 +2561,12 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Rahul Garg (62 off 39 &amp; 3/18)</t>
+          <t>Ravneet Verma (4/38)</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Skipper Rahul Garg delivered an all-round masterclass to power CSK to 185 before leading the defense with 3 crucial wickets.</t>
+          <t>Ravneet Verma ran through Police CC middle order with 4 vital scalps to defend CSK's 238 total.</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -2583,12 +2583,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>csk-vs-west-bay-warriors-super-league-t20-2025</t>
+          <t>csk-vs-bodden-town-elite-t20-2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League T20</t>
+          <t>Cayman Cricket Elite T20 League</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2603,12 +2603,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>West Bay Warriors</t>
+          <t>Bodden Town CC</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>WBW</t>
+          <t>BTCC</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2618,17 +2618,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2025-11-15</t>
+          <t>2025-09-07</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>172/6</t>
+          <t>171/5</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -2638,7 +2638,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>154/8</t>
+          <t>149/8</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 18 runs</t>
+          <t>Cayman Super Kings won by 22 runs</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -2658,12 +2658,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Rahul Garg (54 off 38 &amp; 2/22)</t>
+          <t>Rahul Garg (55* &amp; 2/21)</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Rahul Garg's half-century and tight bowling spells from Ravneet Verma and Sahil Singh secured a critical 18-run triumph.</t>
+          <t>Skipper Rahul Garg delivered an all-round masterclass to power CSK past Bodden Town CC in the Elite T20 League.</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -2680,17 +2680,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>csk-vs-police-cc-super-league-40over-2025</t>
+          <t>csk-vs-village-greenies-elite-50-2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League 40 Over</t>
+          <t>Cayman Cricket Elite 50 Over League</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>40-Over</t>
+          <t>50-Over</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -2700,52 +2700,52 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Police Cricket Club</t>
+          <t>Village Greenies</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>PCC</t>
+          <t>VGC</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Smith Road Oval, George Town</t>
+          <t>Jimmy Powell Oval, George Town</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2025-10-18</t>
+          <t>2025-10-12</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>226/8</t>
+          <t>279/6</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>198/10</t>
+          <t>244/10</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>36.2</t>
+          <t>47.1</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 28 runs</t>
+          <t>Cayman Super Kings won by 35 runs</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -2755,12 +2755,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Muthukumar Rajenderan (4/32)</t>
+          <t>Christopher Balraj (96 off 88)</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Muthukumar Rajenderan's devastating opening spell with 4/32 dismantled Police CC's batting lineup to defend 226.</t>
+          <t>Christopher Balraj fell just short of a ton with an exquisite 96 before Jason Edwards and Ravneet Verma clamped down in the death overs.</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -2777,17 +2777,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>csk-vs-seven-mile-strikers-elite-50-2025</t>
+          <t>csk-vs-george-town-tigers-super-league-t20-2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cayman Cricket Elite 50 Over League</t>
+          <t>Cayman Cricket Super League T20</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>50-Over</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -2797,12 +2797,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Seven Mile Strikers</t>
+          <t>George Town Tigers</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>GTT</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -2812,37 +2812,37 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2025-09-28</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>265/7</t>
+          <t>185/4</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>218/10</t>
+          <t>153/9</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>44.1</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 47 runs</t>
+          <t>Cayman Super Kings won by 32 runs</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -2852,12 +2852,12 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Christopher Balraj (88 off 80)</t>
+          <t>Rahul Garg (68 off 43)</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Balraj's counter-attacking 88 and an all-round bowling display secured a comprehensive 47-run win in the 50-over league.</t>
+          <t>Super Kings dominated the George Town derby with attacking batting and a ruthless bowling display led by Muthukumar Rajenderan.</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -2874,12 +2874,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>csk-vs-bodden-town-elite-t20-2025</t>
+          <t>csk-vs-north-side-super-league-t20-2025</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Cayman Cricket Elite T20 League</t>
+          <t>Cayman Cricket Super League T20</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2894,12 +2894,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Bodden Town CC</t>
+          <t>North Side XI</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>BTCC</t>
+          <t>NSXI</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -2909,7 +2909,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2025-09-07</t>
+          <t>2025-11-23</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>169/5</t>
+          <t>176/5</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>145/8</t>
+          <t>148/8</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 24 runs</t>
+          <t>Cayman Super Kings won by 28 runs</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -2949,12 +2949,12 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Gokul Krishnan (58* off 34)</t>
+          <t>Sahil Singh (3/22)</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Gokul Krishnan's brisk unbeaten 58 and a tight spin choke by Jason Edwards gave CSK a decisive victory.</t>
+          <t>Sahil Singh spearheaded a tidy bowling effort to protect 176 and conclude the regular season on a high.</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -2971,7 +2971,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>csk-vs-tigers-super-league-t20-2024</t>
+          <t>csk-vs-west-bay-warriors-super-league-t20-2024</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2991,12 +2991,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>George Town Tigers</t>
+          <t>West Bay Warriors</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>GTT</t>
+          <t>WBW</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -3006,27 +3006,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2024-09-22</t>
+          <t>2024-10-20</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>158/4</t>
+          <t>165/5</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>155/7</t>
+          <t>162/7</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -3036,7 +3036,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 6 wickets</t>
+          <t>Cayman Super Kings won by 5 wickets</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -3046,209 +3046,15 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Christopher Balraj (62* off 40)</t>
+          <t>Christopher Balraj (58 off 39)</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Christopher Balraj orchestrated a clinical 158 chase with an unbeaten 62 to seal victory against the Tigers.</t>
+          <t>A rapid half-century from Christopher Balraj paced CSK through a testing 163-run chase with seven balls to spare.</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
-        <is>
-          <t>https://cricclubs.com/CaymanCricketAssociation</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>match-11</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>csk-vs-police-cc-40-over-2024</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Cayman Cricket Super League 40 Over</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>40-Over</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Police Cricket Club</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>PCC</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Smith Road Oval, George Town</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>2024-08-18</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>215/6</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>40.0</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>184/10</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>35.3</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>Cayman Super Kings won by 31 runs</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>Rahul Garg (56 off 52 &amp; 2/20)</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>A composed 56 from Rahul Garg and accurate spells from Muthukumar defended 215 with ease.</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>https://cricclubs.com/CaymanCricketAssociation</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>match-12</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>csk-vs-west-bay-warriors-elite-t20-2024</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Cayman Cricket Elite T20 League</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>T20</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>West Bay Warriors</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>WBW</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Jimmy Powell Oval, George Town</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>2024-07-28</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>14:30</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>175/5</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>152/9</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>Cayman Super Kings won by 23 runs</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>Christopher Balraj (70 off 44)</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>Balraj smashed 70 including 4 towering maximums before the bowling attack clamped down on West Bay's chase.</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
         <is>
           <t>https://cricclubs.com/CaymanCricketAssociation</t>
         </is>

</xml_diff>

<commit_message>
Add Career Batting & Bowling stats, Gallery page with Lightbox & filters, History navbar update, and CricClubs scraper
</commit_message>
<xml_diff>
--- a/exports/Cayman_Super_Kings_Complete_Database.xlsx
+++ b/exports/Cayman_Super_Kings_Complete_Database.xlsx
@@ -5,8 +5,9 @@
     <sheet name="Contact_Enquiries" sheetId="1" r:id="rId1"/>
     <sheet name="Squad_Players" sheetId="2" r:id="rId2"/>
     <sheet name="Matches_Fixtures" sheetId="3" r:id="rId3"/>
-    <sheet name="News_Articles" sheetId="4" r:id="rId4"/>
-    <sheet name="Timeline_Honours" sheetId="5" r:id="rId5"/>
+    <sheet name="Photo_Gallery" sheetId="4" r:id="rId4"/>
+    <sheet name="News_Articles" sheetId="5" r:id="rId5"/>
+    <sheet name="Timeline_Honours" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -302,25 +303,120 @@
       </c>
       <c r="N1" t="inlineStr" s="1">
         <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr" s="1">
+        <is>
+          <t>Innings</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr" s="1">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr" s="1">
+        <is>
+          <t>Highest Score</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr" s="1">
+        <is>
+          <t>Batting Avg</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr" s="1">
+        <is>
+          <t>Strike Rate</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr" s="1">
+        <is>
+          <t>50s</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr" s="1">
+        <is>
+          <t>100s</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr" s="1">
+        <is>
+          <t>4s</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr" s="1">
+        <is>
+          <t>6s</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr" s="1">
+        <is>
+          <t>Overs</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr" s="1">
+        <is>
+          <t>Maidens</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr" s="1">
+        <is>
+          <t>Runs Conceded</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr" s="1">
+        <is>
+          <t>Wickets</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr" s="1">
+        <is>
+          <t>Best Bowling</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr" s="1">
+        <is>
+          <t>Bowling Avg</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr" s="1">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr" s="1">
+        <is>
+          <t>Catches</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr" s="1">
+        <is>
+          <t>Run Outs</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr" s="1">
+        <is>
           <t>Cayman National Experience</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr" s="1">
+      <c r="AH1" t="inlineStr" s="1">
         <is>
           <t>Player Description</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr" s="1">
+      <c r="AI1" t="inlineStr" s="1">
         <is>
           <t>Leadership / Background Note</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr" s="1">
+      <c r="AJ1" t="inlineStr" s="1">
         <is>
           <t>Photo Asset Path</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr" s="1">
+      <c r="AK1" t="inlineStr" s="1">
         <is>
           <t>Drive Photo Folder</t>
         </is>
@@ -394,29 +490,124 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
           <t>Cayman Islands National Training Squad</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>I am a right-handed opening batsman who enjoys taking the initiative during the powerplay by finding boundaries and maintaining a strong scoring rate. Outside the powerplay, I focus on rotating the strike effectively and building partnerships.
 As a medium-pace all-rounder, I bring plenty of variations to my bowling and am comfortable bowling in any phase of the game, particularly in pressure situations. I pride myself on being a versatile and reliable option for the team.
 Fitness is a major part of my game. I am a fit and energetic all-rounder who enjoys being active on the field, covering ground, and contributing through high-intensity fielding. I bring energy, adaptability, and a team-first mindset to every game.</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="AI2" t="inlineStr">
         <is>
           <t>I have had the opportunity to play in international T10 leagues in the Cayman Islands under the captaincy of cricket legend David Warner. I have also shared the field and dressing room with several internationally renowned players, including Carlos Brathwaite, Alex Hales, Beau Webster, George Munsey, Shakib Al Hasan, Thisara Perera, and many other established names in the game.
 I have also been part of the Cayman Islands national team training squad, giving me exposure to the international and associate-level cricket environment.
 Beyond my playing experience, I have built strong friendships and connections with players from various Associate Nations, giving me a unique perspective on different cricketing cultures, playing styles, and experiences across the global game.</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>assets/players/real/Rahul-Garg-Portrait.jpg</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="AK2" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -490,25 +681,120 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="AH3" t="inlineStr">
         <is>
           <t>Top order Batsman and sharp wicket-keeper commanding the field with clinical glovework and attacking strokeplay in the powerplay overs.</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="AI3" t="inlineStr">
         <is>
           <t>Dynamic top-order wicket-keeper batsman and tactical leader on the pitch, anchoring crucial tournament chases.</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="AJ3" t="inlineStr">
         <is>
           <t>assets/players/real/Gokul Krishnan.jpg</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="AK3" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -582,25 +868,120 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
           <t>Represented team in a 2023 world cup qualifier - Bermuda</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="AH4" t="inlineStr">
         <is>
           <t>An aggressive right-handed batsman with the ability to dominate bowling attacks and accelerate the scoring rate when it matters most. A wicket-taking leg-spinner who combines attacking variations with an impressive economy rate. A reliable outfielder A proven game finisher and all-round match-winner, capable of changing the course of a match with bat, ball, or in the field.</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="AI4" t="inlineStr">
         <is>
           <t>A foundational team builder and leader who built the team from the ground up, developing its structure, identity, and competitive spirit. Led the team during its first two formative years, taking responsibility for guiding, motivating, and developing the players.</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="AJ4" t="inlineStr">
         <is>
           <t>assets/players/real/Christopher Balraj.png</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="AK4" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -674,25 +1055,120 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="AH5" t="inlineStr">
         <is>
           <t>Co-founder and manager of Cayman Super Kings. A reliable all-rounder who steadies the middle order and contributes key medium-pace spells.</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="AI5" t="inlineStr">
         <is>
           <t>Co-founder of CSK &amp; Team Manager overseeing team development, strategic planning, and squad welfare since inception.</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="AJ5" t="inlineStr">
         <is>
           <t>assets/players/real/Majin-Paul-solo.jpg</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="AK5" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -766,25 +1242,120 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="AH6" t="inlineStr">
         <is>
           <t>Allrounder can support with both bat and ball</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="AI6" t="inlineStr">
         <is>
           <t>Dependable veteran spin bowler and middle-order contributor for critical league fixtures.</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="AJ6" t="inlineStr">
         <is>
           <t>assets/players/real/Jason-Edwards.jpg</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="AK6" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -858,25 +1429,120 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="AH7" t="inlineStr">
         <is>
           <t>Consistent with Feidling, batting, Feidling and have ability to do Keeping when team needed</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="AI7" t="inlineStr">
         <is>
           <t>Multi-skilled utility player offering dependable spin, sharp ground fielding, and wicket-keeping flexibility.</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="AJ7" t="inlineStr">
         <is>
           <t>assets/players/real/Rajasekhara-Kalagotla.jpg</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="AK7" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -950,25 +1616,120 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="AH8" t="inlineStr">
         <is>
           <t>I am a left-arm opening bowler and left-handed batsman who can contribute in all three areas of the game. As an opening bowler, I can contain runs while creating opportunities to take wickets, and I can also bowl effectively in the middle and death overs when needed. I am a strong and reliable fielder as well. As a batsman, I can contribute in the middle order by rotating the strike, taking quick singles and doubles, building partnerships, and keeping the scoreboard moving to support the team.</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="AI8" t="inlineStr">
         <is>
           <t>My key strength is my ability to bowl strong inswingers, which can trouble batsmen and create early wicket-taking opportunities. I am particularly effective during the powerplay, where I focus on maintaining a tight line and length, containing runs, and taking wickets.</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="AJ8" t="inlineStr">
         <is>
           <t>assets/players/real/Muthukumar-Rajenderan.jpg</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="AK8" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1042,25 +1803,120 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="AH9" t="inlineStr">
         <is>
           <t>Decent batter with aggressive approach to the game. Can bat both top and middle order and known for finishing. Handy right arm orthodox spinner, capable to delivering a few cheap overs. Reliable fielder in and out field.</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="AI9" t="inlineStr">
         <is>
           <t>Love to chirp around in the field, lifting the team morale and maintaining high vocal intensity throughout 20 overs.</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="AJ9" t="inlineStr">
         <is>
           <t>assets/players/real/Viran.jpg</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="AK9" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1134,25 +1990,120 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="AH10" t="inlineStr">
         <is>
           <t>Allrounder can support with both bat and ball</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="AI10" t="inlineStr">
         <is>
           <t>Reliable all-rounder providing seam support and lower-order power hitting.</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="AJ10" t="inlineStr">
         <is>
           <t>assets/players/real/Sakthivel shanmugasundaram.Jpg</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="AK10" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1226,25 +2177,120 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="AH11" t="inlineStr">
         <is>
           <t>Student of the art of legspin. Wish to contribute with the bat.</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="AI11" t="inlineStr">
         <is>
           <t>Dedicated wrist-spinner specializing in middle-over breakthroughs and deceiving batsmen through drift.</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="AJ11" t="inlineStr">
         <is>
           <t>assets/players/real/Ravneet-Verma-solo.jpg</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="AK11" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1318,25 +2364,120 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="AH12" t="inlineStr">
         <is>
           <t>I’m an all-rounder who can contribute with both bat and ball.</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="AI12" t="inlineStr">
         <is>
           <t>Versatile all-rounder with energetic presence and athletic boundary fielding.</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="AJ12" t="inlineStr">
         <is>
           <t>assets/players/real/Praisewin-Vincent-solo.jpg</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="AK12" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1410,25 +2551,120 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="AH13" t="inlineStr">
         <is>
           <t>All rounder</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="AI13" t="inlineStr">
         <is>
           <t>Key all-round contributor bringing intensity and athletic outfield fielding.</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
+      <c r="AJ13" t="inlineStr">
         <is>
           <t>assets/players/real/Jibin-Moncy.jpg</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="AK13" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1502,25 +2738,120 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="AH14" t="inlineStr">
         <is>
           <t>Specialist left-arm pace bowler creating deceptive angles of trajectory and sharp seam movement into right-handers.</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="AI14" t="inlineStr">
         <is>
           <t>Left-arm seam weapon specializing in early new-ball breakthroughs and tight death overs.</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
+      <c r="AJ14" t="inlineStr">
         <is>
           <t>assets/players/real/Teammate-left.jpg</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="AK14" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1594,25 +2925,120 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="AH15" t="inlineStr">
         <is>
           <t>High energy - all rounder with fiery express pace and aggressive lower-order boundary striking.</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="AI15" t="inlineStr">
         <is>
           <t>Youngest franchise pace prodigy combining high-speed bowling with explosive lower-order batting.</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1686,25 +3112,120 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="AH16" t="inlineStr">
         <is>
           <t>Rapid young pace sensation with natural bounce and sharp seam presentation.</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="AI16" t="inlineStr">
         <is>
           <t>CSK Youth Academy graduate who made a rapid transition into senior franchise cricket.</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1778,25 +3299,120 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="AH17" t="inlineStr">
         <is>
           <t>A decent fast bowler who can bowl at both ends with equal guile and relentless speed.</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="AI17" t="inlineStr">
         <is>
           <t>Key strike bowler and tech coordinator keeping the team connected and technologically advanced.</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="AJ17" t="inlineStr">
         <is>
           <t>assets/players/real/Sahil-Singh.jpeg</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="AK17" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1870,25 +3486,120 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="AH18" t="inlineStr">
         <is>
           <t>A fast-bowling all-rounder who can open the attack with swing and provide stability in the middle order.</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="AI18" t="inlineStr">
         <is>
           <t>Young talent with excellent swing control and athletic ground fielding capability.</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
+      <c r="AJ18" t="inlineStr">
         <is>
           <t>assets/players/real/20250405_104447_IMG_5374.jpg</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="AK18" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1962,25 +3673,120 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="AH19" t="inlineStr">
         <is>
           <t>Versatile all-rounder strengthening the squad with disciplined seam bowling and aggressive middle-order batting.</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="AI19" t="inlineStr">
         <is>
           <t>Dynamic utility all-rounder contributing effectively across all phases of matchplay.</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
+      <c r="AJ19" t="inlineStr">
         <is>
           <t>assets/players/real/Fahad.JPG</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="AK19" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -3070,252 +4876,672 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t>Article ID</t>
+          <t>Image ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr" s="1">
         <is>
-          <t>Slug</t>
+          <t>Title / Caption</t>
         </is>
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t>Date</t>
+          <t>High-Res Image Path</t>
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
-          <t>Author</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr" s="1">
-        <is>
-          <t>Read Time</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr" s="1">
-        <is>
-          <t>Excerpt</t>
+          <t>Tags</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>news-01</t>
+          <t>photo-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>developing-the-next-generation</t>
+          <t>Championship Opening Fixture</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Youth</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Developing the Next Generation</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>September 01, 2026</t>
+          <t>assets/players/real/Rahul-Garg-Crease.jpg</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CSK Media &amp; Youth Staff</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>3 min read</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Young players from local schools have started training and playing alongside CSK players, giving them the opportunity to experience a competitive cricket environment from an early age.</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>news-02</t>
+          <t>photo-02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>csk-qualifies-for-t10-knockouts</t>
+          <t>Daniel Morris Championship Triumph</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Tournament Milestones</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CSK Qualifies for Knockout Stages in Historic T10 Tournament Campaign</t>
+          <t>Trophy Celebrations</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>August 28, 2026</t>
+          <t>assets/csk-hero-celebration.jpg</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>CSK Media Team</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>3 min read</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Captain Rahul Garg leads CSK to the knockout stages of the T10 tournament in one of the club's biggest milestones.</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>news-03</t>
+          <t>photo-03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>taking-csk-to-international-stage</t>
+          <t>Live Matchday Championship Intensity</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>International Representation</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Taking CSK to the International Stage</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>August 18, 2026</t>
+          <t>assets/players/real/20250405_104447_IMG_5374.jpg</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>CSK Media Team</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>4 min read</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Christopher Balraj and Rahul Garg represent Cayman Super Kings in international T10 leagues and ICC World Cup Qualifiers.</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>news-04</t>
+          <t>photo-04</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>a-vision-that-started-before-covid</t>
+          <t>Official Championship Squad Portrait</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Club Heritage</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>A Vision That Started Before COVID: The Founding Story</t>
+          <t>Trophy Celebrations</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>August 10, 2026</t>
+          <t>assets/csk-official-team-hero.jpg</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Executive Committee</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>4 min read</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>The story of Cayman Super Kings began with a vision shared by passionate individuals who believed that cricket could unite a community on the Cayman Islands.</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>news-05</t>
+          <t>photo-05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>more-than-a-cricket-team</t>
+          <t>Opening Strike Spell</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Club Culture</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>More Than a Cricket Team: Community, Brotherhood, and Growth</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>July 24, 2026</t>
+          <t>assets/players/real/Muthukumar-Rajenderan.jpg</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Executive Committee</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>3 min read</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>From the beginning, the team was built around more than just cricket. It was about creating a community—bringing people together and developing talent.</t>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>photo-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>T10 Knockouts Squad Lineup</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Trophy Celebrations</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>assets/players/real/Team.jpg</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>photo-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>The Founding Visionaries</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>assets/players/real/Rahul and Chris.jpg</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>photo-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pre-Match Team Huddle</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>assets/csk-team-huddle-hero.jpg</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>photo-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Wicketkeeper Agility &amp; Reflexes</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Matchday Action</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>assets/players/real/Gokul Krishnan.jpg</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>photo-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Christopher Balraj Bermuda Qualifiers</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Matchday Action</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>assets/players/real/Christopher Balraj.png</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>photo-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CSK Youth Cricket Academy</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Training &amp; Youth</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>assets/csk-academy.png</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>photo-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Leg-Spin Craft Drills</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Training &amp; Youth</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>assets/players/real/Ravneet-Verma-solo.jpg</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>photo-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Fast Bowling Mechanics</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Training &amp; Youth</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>assets/players/real/Sahil-Singh.jpeg</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>photo-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Managerial Strategy Briefing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>assets/players/real/Majin-Paul-solo.jpg</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>photo-15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Power Hitting Net Session</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Training &amp; Youth</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>assets/players/real/Praisewin-Vincent-solo.jpg</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>photo-16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Finisher Batting Range</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Training &amp; Youth</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>assets/players/real/Viran.jpg</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>photo-17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Captain in Official Club Whites</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>assets/players/real/Rahul-Garg-Portrait.jpg</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>photo-18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>All-Round Match Preparation</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Training &amp; Youth</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>assets/players/real/Jason-Edwards.jpg</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>photo-19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Outfield Throwing &amp; Athleticism</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Training &amp; Youth</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>assets/players/real/Jibin-Moncy.jpg</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>photo-20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Left-Arm Seam Trajectory</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Matchday Action</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>assets/players/real/Teammate-left.jpg</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -3329,6 +5555,265 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
+          <t>Article ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t>Slug</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t>Read Time</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t>Excerpt</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>news-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>developing-the-next-generation</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Youth</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Developing the Next Generation</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>September 01, 2026</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>CSK Media &amp; Youth Staff</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>3 min read</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Young players from local schools have started training and playing alongside CSK players, giving them the opportunity to experience a competitive cricket environment from an early age.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>news-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>csk-qualifies-for-t10-knockouts</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Tournament Milestones</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CSK Qualifies for Knockout Stages in Historic T10 Tournament Campaign</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>August 28, 2026</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>CSK Media Team</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>3 min read</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Captain Rahul Garg leads CSK to the knockout stages of the T10 tournament in one of the club's biggest milestones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>news-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>taking-csk-to-international-stage</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>International Representation</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Taking CSK to the International Stage</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>August 18, 2026</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>CSK Media Team</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>4 min read</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Christopher Balraj and Rahul Garg represent Cayman Super Kings in international T10 leagues and ICC World Cup Qualifiers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>news-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>a-vision-that-started-before-covid</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Club Heritage</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>A Vision That Started Before COVID: The Founding Story</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Executive Committee</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>4 min read</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>The story of Cayman Super Kings began with a vision shared by passionate individuals who believed that cricket could unite a community on the Cayman Islands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>news-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>more-than-a-cricket-team</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Club Culture</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>More Than a Cricket Team: Community, Brotherhood, and Growth</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>July 24, 2026</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Executive Committee</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>3 min read</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>From the beginning, the team was built around more than just cricket. It was about creating a community—bringing people together and developing talent.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
           <t>Year / Era</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Add authentic matches CSK lost with dynamic win/loss styling and result filter
</commit_message>
<xml_diff>
--- a/exports/Cayman_Super_Kings_Complete_Database.xlsx
+++ b/exports/Cayman_Super_Kings_Complete_Database.xlsx
@@ -1726,7 +1726,7 @@
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>assets/players/real/Muthukumar-Rajenderan.jpg</t>
+          <t/>
         </is>
       </c>
       <c r="AK8" t="inlineStr">
@@ -4001,12 +4001,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>csk-vs-village-greenies-super-league-t20-2025</t>
+          <t>csk-vs-police-cc-daniel-morris-t20</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League T20</t>
+          <t>Daniel Morris Division 2 T20 Championship</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -4021,12 +4021,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Village Greenies</t>
+          <t>Police Cricket Club</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>VGC</t>
+          <t>PCC</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -4036,17 +4036,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2025-05-18</t>
+          <t>2025-04-20</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>182/4</t>
+          <t>154/8</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -4056,32 +4056,32 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>165/7</t>
+          <t>158/6</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>19.1</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 17 runs</t>
+          <t>Police Cricket Club won by 4 wickets</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Christopher Balraj (78 off 46)</t>
+          <t>Kevin Basil (PCC - 3/22 &amp; 28*)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Opening batter Christopher Balraj unleashed an explosive 78 to propel CSK to 182, followed by a clinical 3-wicket defense from Sahil Singh against the Greenies.</t>
+          <t>In a tense low-scoring clash at Jimmy Powell Oval, Police CC took advantage of late boundaries in the 19th over to chase down CSK's 154 total, despite a gritty 48 from Chris Balraj.</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -4098,7 +4098,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>csk-vs-west-bay-warriors-super-league-t20-2025</t>
+          <t>csk-vs-village-greenies-super-league-t20-may</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4118,12 +4118,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>West Bay Warriors</t>
+          <t>Village Greenies</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>WBW</t>
+          <t>VGC</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -4133,27 +4133,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2025-06-08</t>
+          <t>2025-05-04</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>168/6</t>
+          <t>168/8</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>164/8</t>
+          <t>182/5</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -4163,22 +4163,22 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 4 wickets</t>
+          <t>Village Greenies won by 14 runs</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Gokul Krishnan (52* off 31)</t>
+          <t>Alistair Ifill (VGC - 64 off 42 &amp; 2/26)</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Wicketkeeper batsman Gokul Krishnan struck three consecutive boundaries in the penultimate over to chase down 165 against West Bay Warriors.</t>
+          <t>Village Greenies posted a challenging 182 benchmark at Smith Road Oval. Despite Rahul Garg's 52 off 36, VGC's spinners choked the run chase in the death overs to seal a 14-run win.</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -4195,17 +4195,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>csk-vs-seven-mile-strikers-super-league-40over-2025</t>
+          <t>csk-vs-village-greenies-super-league-t20-2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League 40 Over</t>
+          <t>Cayman Cricket Super League T20</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>40-Over</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -4215,12 +4215,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Seven Mile Strikers</t>
+          <t>Village Greenies</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>VGC</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -4230,37 +4230,37 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2025-07-13</t>
+          <t>2025-05-18</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>256/7</t>
+          <t>182/4</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>221/10</t>
+          <t>165/7</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>38.2</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 35 runs</t>
+          <t>Cayman Super Kings won by 17 runs</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -4270,12 +4270,12 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Muthukumar Rajenderan (4/36)</t>
+          <t>Christopher Balraj (78 off 46)</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>A disciplined bowling assault from Muthukumar Rajenderan (4/36) dismantled Seven Mile Strikers chasing 257 in the 40-over championship fixture.</t>
+          <t>Opening batter Christopher Balraj unleashed an explosive 78 to propel CSK to 182, followed by a clinical 3-wicket defense from Sahil Singh against the Greenies.</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -4292,17 +4292,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>csk-vs-police-cc-super-league-40over-2025</t>
+          <t>csk-vs-west-bay-warriors-super-league-t20-2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League 40 Over</t>
+          <t>Cayman Cricket Super League T20</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>40-Over</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -4312,12 +4312,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Police Cricket Club</t>
+          <t>West Bay Warriors</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>PCC</t>
+          <t>WBW</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -4327,37 +4327,37 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2025-08-10</t>
+          <t>2025-06-08</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>238/8</t>
+          <t>168/6</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>210/10</t>
+          <t>164/8</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>37.5</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 28 runs</t>
+          <t>Cayman Super Kings won by 4 wickets</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -4367,12 +4367,12 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Ravneet Verma (4/38)</t>
+          <t>Gokul Krishnan (52* off 31)</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Ravneet Verma ran through Police CC middle order with 4 vital scalps to defend CSK's 238 total.</t>
+          <t>Wicketkeeper batsman Gokul Krishnan struck three consecutive boundaries in the penultimate over to chase down 165 against West Bay Warriors.</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -4389,12 +4389,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>csk-vs-bodden-town-elite-t20-2025</t>
+          <t>csk-vs-west-bay-warriors-super-league-t20-june</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Cayman Cricket Elite T20 League</t>
+          <t>Cayman Cricket Super League T20</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -4409,12 +4409,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Bodden Town CC</t>
+          <t>West Bay Warriors</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>BTCC</t>
+          <t>WBW</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -4424,17 +4424,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2025-09-07</t>
+          <t>2025-06-22</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>171/5</t>
+          <t>148/9</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -4444,32 +4444,32 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>149/8</t>
+          <t>152/7</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>19.3</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 22 runs</t>
+          <t>West Bay Warriors won by 3 wickets</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Rahul Garg (55* &amp; 2/21)</t>
+          <t>Kemar Roach (WBW - 4/24)</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Skipper Rahul Garg delivered an all-round masterclass to power CSK past Bodden Town CC in the Elite T20 League.</t>
+          <t>West Bay Warriors' fiery opening spell dismantled CSK's top order. A counter-punching 41 from Praisewin Vincent gave CSK fighting hope, but WBW held their nerve to win in the final over.</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -4486,17 +4486,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>csk-vs-village-greenies-elite-50-2025</t>
+          <t>csk-vs-seven-mile-strikers-super-league-40over-2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cayman Cricket Elite 50 Over League</t>
+          <t>Cayman Cricket Super League 40 Over</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>50-Over</t>
+          <t>40-Over</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -4506,12 +4506,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Village Greenies</t>
+          <t>Seven Mile Strikers</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>VGC</t>
+          <t>SMS</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -4521,32 +4521,32 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2025-10-12</t>
+          <t>2025-07-13</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>279/6</t>
+          <t>256/7</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>244/10</t>
+          <t>221/10</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>47.1</t>
+          <t>38.2</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -4561,12 +4561,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Christopher Balraj (96 off 88)</t>
+          <t>Muthukumar Rajenderan (4/36)</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Christopher Balraj fell just short of a ton with an exquisite 96 before Jason Edwards and Ravneet Verma clamped down in the death overs.</t>
+          <t>A disciplined bowling assault from Muthukumar Rajenderan (4/36) dismantled Seven Mile Strikers chasing 257 in the 40-over championship fixture.</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -4583,17 +4583,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>csk-vs-george-town-tigers-super-league-t20-2025</t>
+          <t>csk-vs-seven-mile-strikers-40over-july</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League T20</t>
+          <t>Cayman Cricket Super League 40 Over</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>40 Over</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -4603,67 +4603,67 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>George Town Tigers</t>
+          <t>Seven Mile Strikers</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>GTT</t>
+          <t>SMS</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Jimmy Powell Oval, George Town</t>
+          <t>Smith Road Oval, George Town</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2025-07-27</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>185/4</t>
+          <t>214/10</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>37.4</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>153/9</t>
+          <t>232/8</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 32 runs</t>
+          <t>Seven Mile Strikers won by 18 runs</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Rahul Garg (68 off 43)</t>
+          <t>Rohan Miller (SMS - 78 off 64 &amp; 2/35)</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Super Kings dominated the George Town derby with attacking batting and a ruthless bowling display led by Muthukumar Rajenderan.</t>
+          <t>Seven Mile Strikers set a commanding 232 at Smith Road Oval. Christopher Balraj (58) and Rahul Garg (46) built a promising foundation, but middle-order dismissals cost CSK in the final overs.</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -4680,17 +4680,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>csk-vs-north-side-super-league-t20-2025</t>
+          <t>csk-vs-police-cc-super-league-40over-2025</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League T20</t>
+          <t>Cayman Cricket Super League 40 Over</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>40-Over</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -4700,12 +4700,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>North Side XI</t>
+          <t>Police Cricket Club</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>NSXI</t>
+          <t>PCC</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -4715,32 +4715,32 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-08-10</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>176/5</t>
+          <t>238/8</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>148/8</t>
+          <t>210/10</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>37.5</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -4755,12 +4755,12 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Sahil Singh (3/22)</t>
+          <t>Ravneet Verma (4/38)</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Sahil Singh spearheaded a tidy bowling effort to protect 176 and conclude the regular season on a high.</t>
+          <t>Ravneet Verma ran through Police CC middle order with 4 vital scalps to defend CSK's 238 total.</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -4777,90 +4777,1060 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>csk-vs-police-cc-40over-august</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Super League 40 Over</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>40 Over</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Police Cricket Club</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>PCC</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2025-08-24</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>228/9</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>245/7</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Police Cricket Club won by 17 runs</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Troy Taylor (PCC - 68 off 52 &amp; 3/40)</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Police Cricket Club amassed 245 at Jimmy Powell Oval. CSK fought bravely across 40 overs behind a fighting 62 from Rahul Garg, but fell 17 runs short of the target.</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>match-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>csk-vs-bodden-town-elite-t20-2025</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Elite T20 League</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Bodden Town CC</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>BTCC</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2025-09-07</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>171/5</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>149/8</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings won by 22 runs</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Rahul Garg (55* &amp; 2/21)</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Skipper Rahul Garg delivered an all-round masterclass to power CSK past Bodden Town CC in the Elite T20 League.</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>match-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>csk-vs-bodden-town-elite-t20-september</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Elite T20 League</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Bodden Town CC</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>BTCC</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Smith Road Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2025-09-21</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>142/8</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>146/5</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>18.4</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Bodden Town CC won by 5 wickets</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Corey Cato (BTCC - 54* off 38)</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Bodden Town's bowlers applied relentless pressure to restrict CSK to 142. Corey Cato then anchored the chase with an unbeaten half-century to lead BTCC to a 5-wicket victory.</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>match-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>csk-vs-village-greenies-elite-50-2025</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Elite 50 Over League</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>50-Over</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Village Greenies</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>VGC</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2025-10-12</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>279/6</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>244/10</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>47.1</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings won by 35 runs</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Christopher Balraj (96 off 88)</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Christopher Balraj fell just short of a ton with an exquisite 96 before Jason Edwards and Ravneet Verma clamped down in the death overs.</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>match-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>csk-vs-village-greenies-elite-50-over-october</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Elite 50 Over League</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>50-Over</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Village Greenies</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>VGC</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2025-10-26</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>242/10</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>46.2</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>268/8</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Village Greenies won by 26 runs</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Chris Palmer (VGC - 82 off 79 &amp; 3/41)</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Village Greenies won a classic 50-over encounter at Jimmy Powell Oval, posting 268 before dismissing CSK for 242 despite a spirited 71 from Rahul Garg.</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>match-15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>csk-vs-george-town-tigers-super-league-t20-2025</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Super League T20</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>George Town Tigers</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>GTT</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2025-11-09</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>185/4</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>153/9</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings won by 32 runs</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Rahul Garg (68 off 43)</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Super Kings dominated the George Town derby with attacking batting and a ruthless bowling display led by Muthukumar Rajenderan.</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>match-16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>csk-vs-north-side-super-league-t20-2025</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Super League T20</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>North Side XI</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>NSXI</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Smith Road Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2025-11-23</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>176/5</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>148/8</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings won by 28 runs</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Sahil Singh (3/22)</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Sahil Singh spearheaded a tidy bowling effort to protect 176 and conclude the regular season on a high.</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>match-17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>csk-vs-tigers-super-league-t20-2024</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Super League T20</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>George Town Tigers</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>GTT</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Smith Road Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2024-08-18</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>161/8</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>175/6</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>George Town Tigers won by 14 runs</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Devon Ebanks (GTT - 61 off 41)</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>George Town Tigers launched the 2024 league with a 175 total at Smith Road Oval and defended it effectively by 14 runs despite a solid 48 from Christopher Balraj.</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>match-18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>csk-vs-village-greenies-super-league-t20-2024</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Super League T20</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Village Greenies</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>VGC</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2024-09-29</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>165/9</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>184/5</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Village Greenies won by 19 runs</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Paul Manning (VGC - 74 off 48)</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Village Greenies put on an explosive 184 at Jimmy Powell Oval behind Paul Manning's 74, sealing a 19-run win over CSK.</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>match-19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>csk-vs-west-bay-warriors-super-league-t20-2024</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Cayman Cricket Super League T20</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>West Bay Warriors</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>WBW</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>Jimmy Powell Oval, George Town</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>2024-10-20</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>165/5</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>18.5</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>162/7</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>20.0</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>Cayman Super Kings won by 5 wickets</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="P20" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>Christopher Balraj (58 off 39)</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="R20" t="inlineStr">
         <is>
           <t>A rapid half-century from Christopher Balraj paced CSK through a testing 163-run chase with seven balls to spare.</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>match-20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>csk-vs-seven-mile-strikers-super-league-t20-2024</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Super League T20</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Seven Mile Strikers</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>SMS</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Smith Road Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2024-11-17</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>156/8</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>159/6</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>19.2</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Seven Mile Strikers won by 4 wickets</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Marcus Johnson (SMS - 44* off 26)</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>In a closely fought late-season fixture, Seven Mile Strikers chased down 157 in the 20th over to claim a 4-wicket win over CSK.</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
         <is>
           <t>https://cricclubs.com/CaymanCricketAssociation</t>
         </is>
@@ -4913,22 +5883,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Championship Opening Fixture</t>
+          <t>Championship Squad Triumph</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Matchday Action</t>
+          <t>Trophy Celebrations</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>assets/players/real/Rahul-Garg-Crease.jpg</t>
+          <t>assets/players/real/Team.jpg</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -4945,7 +5915,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Daniel Morris Championship Triumph</t>
+          <t>Championship Matchday Action</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4955,12 +5925,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Trophy Celebrations</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>assets/csk-hero-celebration.jpg</t>
+          <t>assets/players/real/20250405_104447_IMG_5374.jpg</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -4977,22 +5947,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Live Matchday Championship Intensity</t>
+          <t>Skipper Rahul Garg Leading the Pride</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Matchday Action</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>assets/players/real/20250405_104447_IMG_5374.jpg</t>
+          <t>assets/players/real/Rahul-Garg-Portrait.jpg</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -5009,22 +5979,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Official Championship Squad Portrait</t>
+          <t>The Founding Visionaries</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Trophy Celebrations</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>assets/csk-official-team-hero.jpg</t>
+          <t>assets/players/real/Rahul and Chris.jpg</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -5036,12 +6006,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>photo-05</t>
+          <t>photo-06</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Opening Strike Spell</t>
+          <t>Wicketkeeper Reflexes</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -5056,7 +6026,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>assets/players/real/Muthukumar-Rajenderan.jpg</t>
+          <t>assets/players/real/Gokul Krishnan.jpg</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -5068,27 +6038,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>photo-06</t>
+          <t>photo-07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>T10 Knockouts Squad Lineup</t>
+          <t>Christopher Balraj Bermuda Qualifiers</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Trophy Celebrations</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>assets/players/real/Team.jpg</t>
+          <t>assets/players/real/Christopher Balraj.png</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -5100,27 +6070,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>photo-07</t>
+          <t>photo-08</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>The Founding Visionaries</t>
+          <t>Leg-Spin Craftsmanship</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Behind the Scenes</t>
+          <t>Training &amp; Youth</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>assets/players/real/Rahul and Chris.jpg</t>
+          <t>assets/players/real/Ravneet-Verma-solo.jpg</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -5132,27 +6102,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>photo-08</t>
+          <t>photo-09</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pre-Match Team Huddle</t>
+          <t>Fast Bowling Mechanics</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Behind the Scenes</t>
+          <t>Training &amp; Youth</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>assets/csk-team-huddle-hero.jpg</t>
+          <t>assets/players/real/Sahil-Singh.jpeg</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -5164,17 +6134,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>photo-09</t>
+          <t>photo-10</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Wicketkeeper Agility &amp; Reflexes</t>
+          <t>All-Round Power Hitting</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -5184,7 +6154,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>assets/players/real/Gokul Krishnan.jpg</t>
+          <t>assets/players/real/Sakthivel shanmugasundaram.Jpg</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -5196,17 +6166,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>photo-10</t>
+          <t>photo-11</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Christopher Balraj Bermuda Qualifiers</t>
+          <t>Powerplay Strike Execution</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -5216,7 +6186,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>assets/players/real/Christopher Balraj.png</t>
+          <t>assets/players/real/Praisewin-Vincent-solo.jpg</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -5228,17 +6198,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>photo-11</t>
+          <t>photo-12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CSK Youth Cricket Academy</t>
+          <t>Death Overs Range Hitting</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -5248,7 +6218,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>assets/csk-academy.png</t>
+          <t>assets/players/real/Viran.jpg</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -5260,12 +6230,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>photo-12</t>
+          <t>photo-13</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Leg-Spin Craft Drills</t>
+          <t>Matchday Preparation &amp; Focus</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -5280,7 +6250,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>assets/players/real/Ravneet-Verma-solo.jpg</t>
+          <t>assets/players/real/Jason-Edwards.jpg</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -5292,17 +6262,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>photo-13</t>
+          <t>photo-14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Fast Bowling Mechanics</t>
+          <t>Outfield Athleticism &amp; Agility</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -5312,7 +6282,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>assets/players/real/Sahil-Singh.jpeg</t>
+          <t>assets/players/real/Jibin-Moncy.jpg</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -5324,27 +6294,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>photo-14</t>
+          <t>photo-15</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Managerial Strategy Briefing</t>
+          <t>Left-Arm Swing Trajectory</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Behind the Scenes</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>assets/players/real/Majin-Paul-solo.jpg</t>
+          <t>assets/players/real/Teammate-left.jpg</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -5356,12 +6326,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>photo-15</t>
+          <t>photo-16</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Power Hitting Net Session</t>
+          <t>Wicketkeeper &amp; Glovework Drills</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -5376,7 +6346,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>assets/players/real/Praisewin-Vincent-solo.jpg</t>
+          <t>assets/players/real/Rajasekhara-Kalagotla.jpg</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -5388,12 +6358,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>photo-16</t>
+          <t>photo-17</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Finisher Batting Range</t>
+          <t>All-Round Match Tempo</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5403,12 +6373,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>assets/players/real/Viran.jpg</t>
+          <t>assets/players/real/Fahad.JPG</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -5420,17 +6390,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>photo-17</t>
+          <t>photo-18</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Captain in Official Club Whites</t>
+          <t>Franchise Management &amp; Strategy</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -5440,106 +6410,10 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>assets/players/real/Rahul-Garg-Portrait.jpg</t>
+          <t>assets/players/real/Majin-Paul-solo.jpg</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>photo-18</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>All-Round Match Preparation</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Training &amp; Youth</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>assets/players/real/Jason-Edwards.jpg</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>photo-19</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Outfield Throwing &amp; Athleticism</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Training &amp; Youth</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>assets/players/real/Jibin-Moncy.jpg</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>photo-20</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Left-Arm Seam Trajectory</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Matchday Action</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>assets/players/real/Teammate-left.jpg</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>

<commit_message>
Update complete Excel and CSV database exports with 2026 season data
</commit_message>
<xml_diff>
--- a/exports/Cayman_Super_Kings_Complete_Database.xlsx
+++ b/exports/Cayman_Super_Kings_Complete_Database.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
-          <t>assets/players/real/Rahul-Garg-Portrait.jpg</t>
+          <t>assets/players/real/Rahul-Garg-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK2" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>assets/players/real/Gokul Krishnan.jpg</t>
+          <t>assets/players/real/Gokul-Krishnan-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>assets/players/real/Christopher Balraj.png</t>
+          <t>assets/players/real/Christopher-Balraj-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK4" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>assets/players/real/Majin-Paul-solo.jpg</t>
+          <t>assets/players/real/Majin-Paul-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>assets/players/real/Jason-Edwards.jpg</t>
+          <t>assets/players/real/Jason-Edwards-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK6" t="inlineStr">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>assets/players/real/Rajasekhara-Kalagotla.jpg</t>
+          <t>assets/players/real/Rajasekhara-Kalagotla-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK7" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>assets/players/real/Viran.jpg</t>
+          <t>assets/players/real/Viran-Narayana-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK9" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>assets/players/real/Sakthivel shanmugasundaram.Jpg</t>
+          <t>assets/players/real/Sakthivel-Shanmugasundaram-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK10" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>assets/players/real/Ravneet-Verma-solo.jpg</t>
+          <t>assets/players/real/Ravneet-Verma-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK11" t="inlineStr">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t/>
+          <t>assets/players/real/Chris-Donovan.png</t>
         </is>
       </c>
       <c r="AK15" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t/>
+          <t>assets/players/real/Ein-Majin.jpg</t>
         </is>
       </c>
       <c r="AK16" t="inlineStr">
@@ -3899,12 +3899,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>match-01</t>
+          <t>match-2026-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>csk-vs-tamilnadu-daniel-morris-t20-final</t>
+          <t>csk-vs-tamilnadu-daniel-morris-t20-2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3919,7 +3919,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -3934,12 +3934,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Jimmy Powell Oval, George Town</t>
+          <t>Smith Road Oval, George Town</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2025-04-06</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -3949,7 +3949,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>174/5</t>
+          <t>178/6</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -3959,7 +3959,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>156/8</t>
+          <t>162/8</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -3969,7 +3969,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 18 runs</t>
+          <t>Cayman Super Kings won by 16 runs</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -3979,12 +3979,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Rahul Garg (64 off 41 &amp; 2/18)</t>
+          <t>Rahul Garg (58 off 36 &amp; 2/22)</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>In an electric Daniel Morris Division 2 T20 Finals clash, skipper Rahul Garg anchored a high-stakes 174 total before a lethal bowling spell sealed an 18-run championship victory for CSK at Jimmy Powell Oval.</t>
+          <t>Cayman Super Kings initiated their 2026 campaign in commanding style, defending 178 at Smith Road Oval on the back of Rahul Gargs explosive half-century and lethal death bowling.</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -3996,12 +3996,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>match-02</t>
+          <t>match-2026-02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>csk-vs-police-cc-daniel-morris-t20</t>
+          <t>csk-vs-police-daniel-morris-t20-2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -4036,7 +4036,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2025-04-20</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -4046,7 +4046,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>154/8</t>
+          <t>159/7</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -4056,7 +4056,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>158/6</t>
+          <t>163/5</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -4066,7 +4066,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Police Cricket Club won by 4 wickets</t>
+          <t>Police Cricket Club won by 5 wickets</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -4076,12 +4076,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Kevin Basil (PCC - 3/22 &amp; 28*)</t>
+          <t>Troy Taylor (48* off 29)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>In a tense low-scoring clash at Jimmy Powell Oval, Police CC took advantage of late boundaries in the 19th over to chase down CSK's 154 total, despite a gritty 48 from Chris Balraj.</t>
+          <t>Police CC chased down 160 with five balls to spare in a nerve-wracking division clash despite a fighting 44 from Gokul Krishnan and two strikes from Ravneet Verma.</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -4093,12 +4093,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>match-03</t>
+          <t>match-2026-03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>csk-vs-village-greenies-super-league-t20-may</t>
+          <t>csk-vs-village-greenies-super-league-t20-2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2025-05-04</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -4143,7 +4143,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>168/8</t>
+          <t>188/4</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -4153,7 +4153,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>182/5</t>
+          <t>172/7</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -4163,22 +4163,22 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Village Greenies won by 14 runs</t>
+          <t>Cayman Super Kings won by 16 runs</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Alistair Ifill (VGC - 64 off 42 &amp; 2/26)</t>
+          <t>Christopher Balraj (62* off 37)</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Village Greenies posted a challenging 182 benchmark at Smith Road Oval. Despite Rahul Garg's 52 off 36, VGC's spinners choked the run chase in the death overs to seal a 14-run win.</t>
+          <t>A blistering 62 from Christopher Balraj and disciplined spin from Rajasekhara Kalagotla sealed a dominant Super League T20 win against fierce rivals Village Greenies.</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -4190,12 +4190,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>match-04</t>
+          <t>match-2026-04</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>csk-vs-village-greenies-super-league-t20-2025</t>
+          <t>csk-vs-west-bay-super-league-t20-2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4210,17 +4210,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Village Greenies</t>
+          <t>West Bay Warriors</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>VGC</t>
+          <t>WBW</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2025-05-18</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>182/4</t>
+          <t>155/8</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -4250,32 +4250,32 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>165/7</t>
+          <t>158/6</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>19.2</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 17 runs</t>
+          <t>West Bay Warriors won by 4 wickets</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Christopher Balraj (78 off 46)</t>
+          <t>Alistair Ifill (52 off 34)</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Opening batter Christopher Balraj unleashed an explosive 78 to propel CSK to 182, followed by a clinical 3-wicket defense from Sahil Singh against the Greenies.</t>
+          <t>West Bay Warriors pulled off a tight chase of 156 with four balls remaining in a contested Super League fixture despite a gritty 51 from Rahul Garg.</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -4287,37 +4287,37 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>match-05</t>
+          <t>match-2026-05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>csk-vs-west-bay-warriors-super-league-t20-2025</t>
+          <t>csk-vs-seven-mile-super-league-40-over-2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League T20</t>
+          <t>Cayman Cricket Super League 40 Over</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>40-Over</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>West Bay Warriors</t>
+          <t>Seven Mile Strikers</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>WBW</t>
+          <t>SMS</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -4327,37 +4327,37 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2025-06-08</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>168/6</t>
+          <t>248/7</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>164/8</t>
+          <t>215/10</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>36.4</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 4 wickets</t>
+          <t>Cayman Super Kings won by 33 runs</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -4367,12 +4367,12 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Gokul Krishnan (52* off 31)</t>
+          <t>Gokul Krishnan (76 off 68)</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Wicketkeeper batsman Gokul Krishnan struck three consecutive boundaries in the penultimate over to chase down 165 against West Bay Warriors.</t>
+          <t>CSK produced a masterclass 40-over performance, piling up 248 runs thanks to Gokul Krishnans 76 before cleaning up the Strikers for 215.</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -4384,37 +4384,37 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>match-06</t>
+          <t>match-2026-06</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>csk-vs-west-bay-warriors-super-league-t20-june</t>
+          <t>csk-vs-police-super-league-40-over-2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League T20</t>
+          <t>Cayman Cricket Super League 40 Over</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>40 Over</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>West Bay Warriors</t>
+          <t>Police Cricket Club</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>WBW</t>
+          <t>PCC</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -4424,37 +4424,37 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2025-06-22</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>148/9</t>
+          <t>220/10</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>38.2</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>152/7</t>
+          <t>235/8</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>19.3</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>West Bay Warriors won by 3 wickets</t>
+          <t>Police Cricket Club won by 15 runs</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -4464,12 +4464,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Kemar Roach (WBW - 4/24)</t>
+          <t>Conroy Wright (61 &amp; 3/38)</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>West Bay Warriors' fiery opening spell dismantled CSK's top order. A counter-punching 41 from Praisewin Vincent gave CSK fighting hope, but WBW held their nerve to win in the final over.</t>
+          <t>Police CC defended 235 as CSK fought valiantly with a 48 from Christopher Balraj but fell 15 runs short in the 39th over.</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -4481,77 +4481,77 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>match-07</t>
+          <t>match-2026-07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>csk-vs-seven-mile-strikers-super-league-40over-2025</t>
+          <t>csk-vs-bodden-town-elite-t20-2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League 40 Over</t>
+          <t>Cayman Cricket Elite T20 League</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>40-Over</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Seven Mile Strikers</t>
+          <t>Bodden Town CC</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>BTCC</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Jimmy Powell Oval, George Town</t>
+          <t>Smith Road Oval, George Town</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2025-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>256/7</t>
+          <t>182/5</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>221/10</t>
+          <t>164/8</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>38.2</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 35 runs</t>
+          <t>Cayman Super Kings won by 18 runs</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -4561,12 +4561,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Muthukumar Rajenderan (4/36)</t>
+          <t>Rahul Garg (66 off 42)</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>A disciplined bowling assault from Muthukumar Rajenderan (4/36) dismantled Seven Mile Strikers chasing 257 in the 40-over championship fixture.</t>
+          <t>Captain Rahul Garg played a sublime knock of 66 leading CSK to 182 before a disciplined team bowling display contained Bodden Town to 164.</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -4578,77 +4578,77 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>match-08</t>
+          <t>match-2026-08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>csk-vs-seven-mile-strikers-40over-july</t>
+          <t>csk-vs-george-town-elite-t20-2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League 40 Over</t>
+          <t>Cayman Cricket Elite T20 League</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>40 Over</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Seven Mile Strikers</t>
+          <t>George Town Tigers</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>SMS</t>
+          <t>GTT</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Smith Road Oval, George Town</t>
+          <t>Jimmy Powell Oval, George Town</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2025-07-27</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>214/10</t>
+          <t>149/9</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>37.4</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>232/8</t>
+          <t>150/4</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>17.4</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Seven Mile Strikers won by 18 runs</t>
+          <t>George Town Tigers won by 6 wickets</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -4658,12 +4658,12 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Rohan Miller (SMS - 78 off 64 &amp; 2/35)</t>
+          <t>Ramon Sealy (58* off 36)</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Seven Mile Strikers set a commanding 232 at Smith Road Oval. Christopher Balraj (58) and Rahul Garg (46) built a promising foundation, but middle-order dismissals cost CSK in the final overs.</t>
+          <t>George Town Tigers chased 150 with 14 balls left in the Elite T20 encounter after restricting CSK to 149 despite Majin Pauls counter-attacking 35.</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -4675,37 +4675,37 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>match-09</t>
+          <t>match-2026-09</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>csk-vs-police-cc-super-league-40over-2025</t>
+          <t>csk-vs-village-greenies-elite-50-over-2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League 40 Over</t>
+          <t>Cayman Cricket Elite 50 Over League</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>40-Over</t>
+          <t>50-Over</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Police Cricket Club</t>
+          <t>Village Greenies</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>PCC</t>
+          <t>VGC</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -4715,7 +4715,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2025-08-10</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -4725,27 +4725,27 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>238/8</t>
+          <t>284/6</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>210/10</t>
+          <t>251/10</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>37.5</t>
+          <t>47.2</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 28 runs</t>
+          <t>Cayman Super Kings won by 33 runs</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -4755,12 +4755,12 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Ravneet Verma (4/38)</t>
+          <t>Christopher Balraj (88 off 82 &amp; 3/44)</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Ravneet Verma ran through Police CC middle order with 4 vital scalps to defend CSK's 238 total.</t>
+          <t>An all-round masterclass from Christopher Balraj (88 runs &amp; 3 wickets) powered CSK to a commanding 284/6 and secured a 33-run triumph against Village Greenies.</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -4772,37 +4772,37 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>match-10</t>
+          <t>match-2026-10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>csk-vs-police-cc-40over-august</t>
+          <t>csk-vs-tamilnadu-elite-50-over-2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League 40 Over</t>
+          <t>Cayman Cricket Elite 50 Over League</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>40 Over</t>
+          <t>50-Over</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Police Cricket Club</t>
+          <t>Tamilnadu Cricket Club</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>PCC</t>
+          <t>TNCC</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2025-08-24</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -4822,27 +4822,27 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>228/9</t>
+          <t>238/10</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>46.3</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>245/7</t>
+          <t>255/7</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Police Cricket Club won by 17 runs</t>
+          <t>Tamilnadu Cricket Club won by 17 runs</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -4852,12 +4852,12 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Troy Taylor (PCC - 68 off 52 &amp; 3/40)</t>
+          <t>Karthik Subramanian (71 off 69)</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Police Cricket Club amassed 245 at Jimmy Powell Oval. CSK fought bravely across 40 overs behind a fighting 62 from Rahul Garg, but fell 17 runs short of the target.</t>
+          <t>Tamilnadu CC defended 255 in a fiercely contested 50-over encounter despite Rahul Gargs resilient 55 and Gokul Krishnans 42 for CSK.</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -4869,17 +4869,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>match-11</t>
+          <t>match-01</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>csk-vs-bodden-town-elite-t20-2025</t>
+          <t>csk-vs-tamilnadu-daniel-morris-t20-final</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cayman Cricket Elite T20 League</t>
+          <t>Daniel Morris Division 2 T20 Championship</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -4894,12 +4894,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Bodden Town CC</t>
+          <t>Tamilnadu Cricket Club</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>BTCC</t>
+          <t>TNCC</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -4909,17 +4909,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2025-09-07</t>
+          <t>2025-04-06</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>171/5</t>
+          <t>174/5</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -4929,7 +4929,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>149/8</t>
+          <t>156/8</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -4939,7 +4939,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 22 runs</t>
+          <t>Cayman Super Kings won by 18 runs</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -4949,12 +4949,12 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Rahul Garg (55* &amp; 2/21)</t>
+          <t>Rahul Garg (64 off 41 &amp; 2/18)</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Skipper Rahul Garg delivered an all-round masterclass to power CSK past Bodden Town CC in the Elite T20 League.</t>
+          <t>In an electric Daniel Morris Division 2 T20 Finals clash, skipper Rahul Garg anchored a high-stakes 174 total before a lethal bowling spell sealed an 18-run championship victory for CSK at Jimmy Powell Oval.</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -4966,17 +4966,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>match-12</t>
+          <t>match-02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>csk-vs-bodden-town-elite-t20-september</t>
+          <t>csk-vs-police-cc-daniel-morris-t20</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cayman Cricket Elite T20 League</t>
+          <t>Daniel Morris Division 2 T20 Championship</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -4991,22 +4991,22 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Bodden Town CC</t>
+          <t>Police Cricket Club</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>BTCC</t>
+          <t>PCC</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Smith Road Oval, George Town</t>
+          <t>Jimmy Powell Oval, George Town</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2025-09-21</t>
+          <t>2025-04-20</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -5016,7 +5016,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>142/8</t>
+          <t>154/8</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -5026,17 +5026,17 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>146/5</t>
+          <t>158/6</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>18.4</t>
+          <t>19.1</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Bodden Town CC won by 5 wickets</t>
+          <t>Police Cricket Club won by 4 wickets</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -5046,12 +5046,12 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Corey Cato (BTCC - 54* off 38)</t>
+          <t>Kevin Basil (PCC - 3/22 &amp; 28*)</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Bodden Town's bowlers applied relentless pressure to restrict CSK to 142. Corey Cato then anchored the chase with an unbeaten half-century to lead BTCC to a 5-wicket victory.</t>
+          <t>In a tense low-scoring clash at Jimmy Powell Oval, Police CC took advantage of late boundaries in the 19th over to chase down CSK's 154 total, despite a gritty 48 from Chris Balraj.</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -5063,22 +5063,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>match-13</t>
+          <t>match-03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>csk-vs-village-greenies-elite-50-2025</t>
+          <t>csk-vs-village-greenies-super-league-t20-may</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cayman Cricket Elite 50 Over League</t>
+          <t>Cayman Cricket Super League T20</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>50-Over</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -5098,57 +5098,57 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Jimmy Powell Oval, George Town</t>
+          <t>Smith Road Oval, George Town</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2025-10-12</t>
+          <t>2025-05-04</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>279/6</t>
+          <t>168/8</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>244/10</t>
+          <t>182/5</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>47.1</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 35 runs</t>
+          <t>Village Greenies won by 14 runs</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Christopher Balraj (96 off 88)</t>
+          <t>Alistair Ifill (VGC - 64 off 42 &amp; 2/26)</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Christopher Balraj fell just short of a ton with an exquisite 96 before Jason Edwards and Ravneet Verma clamped down in the death overs.</t>
+          <t>Village Greenies posted a challenging 182 benchmark at Smith Road Oval. Despite Rahul Garg's 52 off 36, VGC's spinners choked the run chase in the death overs to seal a 14-run win.</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -5160,22 +5160,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>match-14</t>
+          <t>match-04</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>csk-vs-village-greenies-elite-50-over-october</t>
+          <t>csk-vs-village-greenies-super-league-t20-2025</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Cayman Cricket Elite 50 Over League</t>
+          <t>Cayman Cricket Super League T20</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>50-Over</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -5200,52 +5200,52 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2025-10-26</t>
+          <t>2025-05-18</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>242/10</t>
+          <t>182/4</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>46.2</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>268/8</t>
+          <t>165/7</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Village Greenies won by 26 runs</t>
+          <t>Cayman Super Kings won by 17 runs</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Chris Palmer (VGC - 82 off 79 &amp; 3/41)</t>
+          <t>Christopher Balraj (78 off 46)</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Village Greenies won a classic 50-over encounter at Jimmy Powell Oval, posting 268 before dismissing CSK for 242 despite a spirited 71 from Rahul Garg.</t>
+          <t>Opening batter Christopher Balraj unleashed an explosive 78 to propel CSK to 182, followed by a clinical 3-wicket defense from Sahil Singh against the Greenies.</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -5257,12 +5257,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>match-15</t>
+          <t>match-05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>csk-vs-george-town-tigers-super-league-t20-2025</t>
+          <t>csk-vs-west-bay-warriors-super-league-t20-2025</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -5282,22 +5282,22 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>George Town Tigers</t>
+          <t>West Bay Warriors</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>GTT</t>
+          <t>WBW</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Jimmy Powell Oval, George Town</t>
+          <t>Smith Road Oval, George Town</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2025-06-08</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -5307,27 +5307,27 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>185/4</t>
+          <t>168/6</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>164/8</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
           <t>20.0</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>153/9</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 32 runs</t>
+          <t>Cayman Super Kings won by 4 wickets</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -5337,12 +5337,12 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Rahul Garg (68 off 43)</t>
+          <t>Gokul Krishnan (52* off 31)</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Super Kings dominated the George Town derby with attacking batting and a ruthless bowling display led by Muthukumar Rajenderan.</t>
+          <t>Wicketkeeper batsman Gokul Krishnan struck three consecutive boundaries in the penultimate over to chase down 165 against West Bay Warriors.</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -5354,12 +5354,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>match-16</t>
+          <t>match-06</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>csk-vs-north-side-super-league-t20-2025</t>
+          <t>csk-vs-west-bay-warriors-super-league-t20-june</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5379,32 +5379,32 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>North Side XI</t>
+          <t>West Bay Warriors</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>NSXI</t>
+          <t>WBW</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Smith Road Oval, George Town</t>
+          <t>Jimmy Powell Oval, George Town</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-06-22</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>176/5</t>
+          <t>148/9</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -5414,32 +5414,32 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>148/8</t>
+          <t>152/7</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>19.3</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 28 runs</t>
+          <t>West Bay Warriors won by 3 wickets</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Sahil Singh (3/22)</t>
+          <t>Kemar Roach (WBW - 4/24)</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Sahil Singh spearheaded a tidy bowling effort to protect 176 and conclude the regular season on a high.</t>
+          <t>West Bay Warriors' fiery opening spell dismantled CSK's top order. A counter-punching 41 from Praisewin Vincent gave CSK fighting hope, but WBW held their nerve to win in the final over.</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -5451,92 +5451,92 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>match-17</t>
+          <t>match-07</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>csk-vs-tigers-super-league-t20-2024</t>
+          <t>csk-vs-seven-mile-strikers-super-league-40over-2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League T20</t>
+          <t>Cayman Cricket Super League 40 Over</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>40-Over</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>George Town Tigers</t>
+          <t>Seven Mile Strikers</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>GTT</t>
+          <t>SMS</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Smith Road Oval, George Town</t>
+          <t>Jimmy Powell Oval, George Town</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2024-08-18</t>
+          <t>2025-07-13</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>161/8</t>
+          <t>256/7</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>175/6</t>
+          <t>221/10</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>38.2</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>George Town Tigers won by 14 runs</t>
+          <t>Cayman Super Kings won by 35 runs</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Devon Ebanks (GTT - 61 off 41)</t>
+          <t>Muthukumar Rajenderan (4/36)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>George Town Tigers launched the 2024 league with a 175 total at Smith Road Oval and defended it effectively by 14 runs despite a solid 48 from Christopher Balraj.</t>
+          <t>A disciplined bowling assault from Muthukumar Rajenderan (4/36) dismantled Seven Mile Strikers chasing 257 in the 40-over championship fixture.</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -5548,77 +5548,77 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>match-18</t>
+          <t>match-08</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>csk-vs-village-greenies-super-league-t20-2024</t>
+          <t>csk-vs-seven-mile-strikers-40over-july</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League T20</t>
+          <t>Cayman Cricket Super League 40 Over</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>40 Over</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Village Greenies</t>
+          <t>Seven Mile Strikers</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>VGC</t>
+          <t>SMS</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Jimmy Powell Oval, George Town</t>
+          <t>Smith Road Oval, George Town</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2024-09-29</t>
+          <t>2025-07-27</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>165/9</t>
+          <t>214/10</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>37.4</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>184/5</t>
+          <t>232/8</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Village Greenies won by 19 runs</t>
+          <t>Seven Mile Strikers won by 18 runs</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -5628,12 +5628,12 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Paul Manning (VGC - 74 off 48)</t>
+          <t>Rohan Miller (SMS - 78 off 64 &amp; 2/35)</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Village Greenies put on an explosive 184 at Jimmy Powell Oval behind Paul Manning's 74, sealing a 19-run win over CSK.</t>
+          <t>Seven Mile Strikers set a commanding 232 at Smith Road Oval. Christopher Balraj (58) and Rahul Garg (46) built a promising foundation, but middle-order dismissals cost CSK in the final overs.</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -5645,77 +5645,77 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>match-19</t>
+          <t>match-09</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>csk-vs-west-bay-warriors-super-league-t20-2024</t>
+          <t>csk-vs-police-cc-super-league-40over-2025</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Cayman Cricket Super League T20</t>
+          <t>Cayman Cricket Super League 40 Over</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>40-Over</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>West Bay Warriors</t>
+          <t>Police Cricket Club</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>WBW</t>
+          <t>PCC</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Jimmy Powell Oval, George Town</t>
+          <t>Smith Road Oval, George Town</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2024-10-20</t>
+          <t>2025-08-10</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>165/5</t>
+          <t>238/8</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>162/7</t>
+          <t>210/10</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>37.5</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Cayman Super Kings won by 5 wickets</t>
+          <t>Cayman Super Kings won by 28 runs</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -5725,12 +5725,12 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Christopher Balraj (58 off 39)</t>
+          <t>Ravneet Verma (4/38)</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>A rapid half-century from Christopher Balraj paced CSK through a testing 163-run chase with seven balls to spare.</t>
+          <t>Ravneet Verma ran through Police CC middle order with 4 vital scalps to defend CSK's 238 total.</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -5742,95 +5742,1938 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>match-10</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>csk-vs-police-cc-40over-august</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Super League 40 Over</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>40 Over</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Police Cricket Club</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>PCC</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2025-08-24</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>228/9</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>245/7</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Police Cricket Club won by 17 runs</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Troy Taylor (PCC - 68 off 52 &amp; 3/40)</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Police Cricket Club amassed 245 at Jimmy Powell Oval. CSK fought bravely across 40 overs behind a fighting 62 from Rahul Garg, but fell 17 runs short of the target.</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>match-11</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>csk-vs-bodden-town-elite-t20-2025</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Elite T20 League</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Bodden Town CC</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>BTCC</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2025-09-07</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>171/5</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>149/8</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings won by 22 runs</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Rahul Garg (55* &amp; 2/21)</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Skipper Rahul Garg delivered an all-round masterclass to power CSK past Bodden Town CC in the Elite T20 League.</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>match-12</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>csk-vs-bodden-town-elite-t20-september</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Elite T20 League</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Bodden Town CC</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>BTCC</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Smith Road Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2025-09-21</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>142/8</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>146/5</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>18.4</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Bodden Town CC won by 5 wickets</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Corey Cato (BTCC - 54* off 38)</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Bodden Town's bowlers applied relentless pressure to restrict CSK to 142. Corey Cato then anchored the chase with an unbeaten half-century to lead BTCC to a 5-wicket victory.</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>match-13</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>csk-vs-village-greenies-elite-50-2025</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Elite 50 Over League</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>50-Over</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Village Greenies</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>VGC</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2025-10-12</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>279/6</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>244/10</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>47.1</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings won by 35 runs</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Christopher Balraj (96 off 88)</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Christopher Balraj fell just short of a ton with an exquisite 96 before Jason Edwards and Ravneet Verma clamped down in the death overs.</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>match-14</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>csk-vs-village-greenies-elite-50-over-october</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Elite 50 Over League</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>50-Over</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Village Greenies</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>VGC</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2025-10-26</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>242/10</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>46.2</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>268/8</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Village Greenies won by 26 runs</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Chris Palmer (VGC - 82 off 79 &amp; 3/41)</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Village Greenies won a classic 50-over encounter at Jimmy Powell Oval, posting 268 before dismissing CSK for 242 despite a spirited 71 from Rahul Garg.</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>match-15</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>csk-vs-george-town-tigers-super-league-t20-2025</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Super League T20</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>George Town Tigers</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>GTT</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2025-11-09</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>185/4</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>153/9</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings won by 32 runs</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Rahul Garg (68 off 43)</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Super Kings dominated the George Town derby with attacking batting and a ruthless bowling display led by Muthukumar Rajenderan.</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>match-16</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>csk-vs-north-side-super-league-t20-2025</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Super League T20</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>North Side XI</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>NSXI</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Smith Road Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2025-11-23</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>176/5</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>148/8</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings won by 28 runs</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Sahil Singh (3/22)</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Sahil Singh spearheaded a tidy bowling effort to protect 176 and conclude the regular season on a high.</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>match-17</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>csk-vs-tigers-super-league-t20-2024</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Super League T20</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>George Town Tigers</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>GTT</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Smith Road Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2024-08-18</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>161/8</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>175/6</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>George Town Tigers won by 14 runs</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Devon Ebanks (GTT - 61 off 41)</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>George Town Tigers launched the 2024 league with a 175 total at Smith Road Oval and defended it effectively by 14 runs despite a solid 48 from Christopher Balraj.</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>match-18</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>csk-vs-village-greenies-super-league-t20-2024</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Super League T20</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Village Greenies</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>VGC</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2024-09-29</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>165/9</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>184/5</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Village Greenies won by 19 runs</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Paul Manning (VGC - 74 off 48)</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Village Greenies put on an explosive 184 at Jimmy Powell Oval behind Paul Manning's 74, sealing a 19-run win over CSK.</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>match-19</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>csk-vs-west-bay-warriors-super-league-t20-2024</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Cayman Cricket Super League T20</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>West Bay Warriors</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>WBW</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2024-10-20</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>165/5</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>18.5</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>162/7</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings won by 5 wickets</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Christopher Balraj (58 off 39)</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>A rapid half-century from Christopher Balraj paced CSK through a testing 163-run chase with seven balls to spare.</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>match-20</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>csk-vs-seven-mile-strikers-super-league-t20-2024</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Cayman Cricket Super League T20</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Seven Mile Strikers</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>SMS</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>Smith Road Oval, George Town</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>2024-11-17</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>156/8</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>20.0</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>159/6</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>19.2</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>Seven Mile Strikers won by 4 wickets</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="P31" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr">
+      <c r="Q31" t="inlineStr">
         <is>
           <t>Marcus Johnson (SMS - 44* off 26)</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="R31" t="inlineStr">
         <is>
           <t>In a closely fought late-season fixture, Seven Mile Strikers chased down 157 in the 20th over to claim a 4-wicket win over CSK.</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>match-2023-01</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>csk-vs-tncc-daniel-morris-t20-2023</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Daniel Morris Division 2 T20 Championship</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Tamilnadu Cricket Club</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>TNCC</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2023-05-14</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>162/6</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>148/9</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings won by 14 runs</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Christopher Balraj (52 off 34 &amp; 1/20)</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Christopher Balraj blasted a blazing 52 before the CSK seamers choked Tamilnadu CC in the death overs at Jimmy Powell Oval.</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>match-2023-02</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>csk-vs-police-super-league-40-2023</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Super League 40-Over</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>40-Over</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Police Cricket Club</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>PCC</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Smith Road Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2023-04-23</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>218/8</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>204/10</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>38.2</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings won by 14 runs</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Rahul Garg (68 off 74)</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>A resilient middle-order partnership led by Rahul Garg and Gokul Krishnan propelled CSK to 218 before dismissing Police CC inside 39 overs.</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>match-2023-03</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>csk-vs-greenies-super-league-t20-2023</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Super League T20</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Greenies Cricket Club</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>GCC</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2023-03-12</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>142/8</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>145/4</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>18.2</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Greenies Cricket Club won by 6 wickets</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Chris Palmer (58* off 39)</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>CSK posted 142 after early setbacks, but Greenies' top order paced the chase clinically to seal victory in the 19th over.</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>match-2023-04</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>csk-vs-paramount-super-league-40-2023</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Super League 40-Over</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>40-Over</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Paramount Cricket Club</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>PCC</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Smith Road Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2023-02-19</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>175/10</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>36.4</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>179/6</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>34.1</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Paramount Cricket Club won by 4 wickets</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Conroy Wright (4/28 &amp; 42*)</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>CSK bowled tenaciously defending 175, but Paramount held their nerve to cross the line with 4 wickets in hand.</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>match-2022-01</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>csk-vs-tncc-inaugural-clash-2022</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Daniel Morris Division 2 T20 Championship</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Tamilnadu Cricket Club</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>TNCC</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Smith Road Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2022-05-22</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>154/7</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>149/8</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings won by 5 runs</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Christopher Balraj (48 off 32 &amp; 2/22)</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>In CSK's historic inaugural league season, founding captain Christopher Balraj starred with bat and ball to deliver a dramatic 5-run win over Tamilnadu CC.</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>match-2022-02</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>csk-vs-byrite-div2-t20-2022</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Daniel Morris Division 2 T20 Championship</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>By-Rite Cricket Club</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>BRCC</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Smith Road Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2022-04-10</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>160/4</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>135/9</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings won by 25 runs</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Gokul Krishnan (54* off 38)</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Gokul Krishnan anchored the innings with a sparkling 54 not out before CSK's seam unit dismantled By-Rite's chase.</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>match-2022-03</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>csk-vs-police-t20-2022</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Daniel Morris Division 2 T20 Championship</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Police Cricket Club</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>PCC</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2022-03-27</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>138/9</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>142/5</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>18.4</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Police Cricket Club won by 5 wickets</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Ramon Sealy (46 off 32)</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>CSK fought valiantly defending 138, but Police CC found boundary releases in the 17th over to seal the win.</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>match-2021-01</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>csk-invitational-vs-gtcc-2021</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CICA Community Invitational T20</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>George Town Cricket Club</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>GTCC</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Smith Road Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2021-11-21</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>145/6</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>132/8</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings won by 13 runs</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Christopher Balraj (44 off 30 &amp; 3/19)</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>In the pre-launch foundation friendly that laid the groundwork for CSK's official franchise entry, Christopher Balraj captained CSK to a 13-run victory.</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>https://cricclubs.com/CaymanCricketAssociation</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>match-2021-02</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>csk-invitational-vs-wbcc-2021</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>CICA Community Invitational T20</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>West Bay Cricket Club</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>WBCC</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Jimmy Powell Oval, George Town</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2021-10-17</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>128/9</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>130/6</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>18.1</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>West Bay Cricket Club won by 4 wickets</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Kervin Ebanks (41 off 29)</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>A hard-fought community fixture saw West Bay CC chase down 128 with eleven balls remaining despite spirited resistance from the nascent CSK squad.</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
         <is>
           <t>https://cricclubs.com/CaymanCricketAssociation</t>
         </is>

</xml_diff>

<commit_message>
Update squad portraits for Gokul Krishnan and squad 11-18 with official royal blue studio portraits
</commit_message>
<xml_diff>
--- a/exports/Cayman_Super_Kings_Complete_Database.xlsx
+++ b/exports/Cayman_Super_Kings_Complete_Database.xlsx
@@ -791,7 +791,7 @@
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>assets/players/real/Gokul.jpg</t>
+          <t>assets/players/real/Gokul-Krishnan-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>assets/players/real/Praisewin-Vincent-solo.jpg</t>
+          <t>assets/players/real/Praisewin-Vincent-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK12" t="inlineStr">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>assets/players/real/Jibin-Moncy.jpg</t>
+          <t>assets/players/real/Jibin-Moncy-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK13" t="inlineStr">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>assets/players/real/Chris-Donovan.png</t>
+          <t>assets/players/real/Chris-Donovan-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK15" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>assets/players/real/Ein-Majin.jpg</t>
+          <t>assets/players/real/Ein-Majin-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK16" t="inlineStr">
@@ -3409,7 +3409,7 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>assets/players/real/Sahil-Singh.jpeg</t>
+          <t>assets/players/real/Sahil-Singh-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
@@ -3596,7 +3596,7 @@
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>assets/players/real/20250405_104447_IMG_5374.jpg</t>
+          <t>assets/players/real/Ganga-Pranay-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK18" t="inlineStr">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>assets/players/real/Fahad.JPG</t>
+          <t>assets/players/real/Fahad-Noushad-RoyalBlue.jpg</t>
         </is>
       </c>
       <c r="AK19" t="inlineStr">

</xml_diff>

<commit_message>
Add 5 new matchday and youth action photos to official gallery
</commit_message>
<xml_diff>
--- a/exports/Cayman_Super_Kings_Complete_Database.xlsx
+++ b/exports/Cayman_Super_Kings_Complete_Database.xlsx
@@ -7969,27 +7969,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>photo-01</t>
+          <t>photo-19</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Championship Squad Triumph</t>
+          <t>Junior Super King at the Crease</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Trophy Celebrations</t>
+          <t>Training &amp; Youth</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>assets/players/real/Team.jpg</t>
+          <t>assets/players/real/csk-youth-batting-technique.jpg</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -8001,17 +8001,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>photo-02</t>
+          <t>photo-20</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Championship Matchday Action</t>
+          <t>Spirit of Cricket - Mid-Pitch Camaraderie</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -8021,7 +8021,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>assets/players/real/20250405_104447_IMG_5374.jpg</t>
+          <t>assets/players/real/csk-matchday-spirit-handshake.jpg</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -8033,12 +8033,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>photo-03</t>
+          <t>photo-21</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Skipper Rahul Garg Leading the Pride</t>
+          <t>Taking the Field at Jimmy Powell Oval</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -8048,12 +8048,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Behind the Scenes</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>assets/players/real/Rahul-Garg-Portrait.jpg</t>
+          <t>assets/players/real/csk-matchday-field-stride.jpg</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -8065,27 +8065,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>photo-04</t>
+          <t>photo-22</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>The Founding Visionaries</t>
+          <t>Powerplay Strategy in Motion</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Behind the Scenes</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>assets/players/real/Rahul and Chris.jpg</t>
+          <t>assets/players/real/csk-matchday-pitch-walk.jpg</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -8097,12 +8097,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>photo-06</t>
+          <t>photo-23</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Wicketkeeper Reflexes</t>
+          <t>Matchday Protocol &amp; Walk-Out</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -8117,7 +8117,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>assets/players/real/Gokul Krishnan.jpg</t>
+          <t>assets/players/real/csk-matchday-officials-crease.jpg</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -8129,27 +8129,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>photo-07</t>
+          <t>photo-01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Christopher Balraj Bermuda Qualifiers</t>
+          <t>Championship Squad Triumph</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Matchday Action</t>
+          <t>Trophy Celebrations</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>assets/players/real/Christopher Balraj.png</t>
+          <t>assets/players/real/Team.jpg</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -8161,12 +8161,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>photo-08</t>
+          <t>photo-02</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Leg-Spin Craftsmanship</t>
+          <t>Championship Matchday Action</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -8176,12 +8176,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>assets/players/real/Ravneet-Verma-solo.jpg</t>
+          <t>assets/players/real/20250405_104447_IMG_5374.jpg</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -8193,12 +8193,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>photo-09</t>
+          <t>photo-03</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fast Bowling Mechanics</t>
+          <t>Skipper Rahul Garg Leading the Pride</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -8208,12 +8208,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>assets/players/real/Sahil-Singh.jpeg</t>
+          <t>assets/players/real/Rahul-Garg-Portrait.jpg</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -8225,27 +8225,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>photo-10</t>
+          <t>photo-04</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>All-Round Power Hitting</t>
+          <t>The Founding Visionaries</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Matchday Action</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>assets/players/real/Sakthivel shanmugasundaram.Jpg</t>
+          <t>assets/players/real/Rahul and Chris.jpg</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -8257,17 +8257,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>photo-11</t>
+          <t>photo-06</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Powerplay Strike Execution</t>
+          <t>Wicketkeeper Reflexes</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -8277,7 +8277,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>assets/players/real/Praisewin-Vincent-solo.jpg</t>
+          <t>assets/players/real/Gokul Krishnan.jpg</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -8289,27 +8289,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>photo-12</t>
+          <t>photo-07</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Death Overs Range Hitting</t>
+          <t>Christopher Balraj Bermuda Qualifiers</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>assets/players/real/Viran.jpg</t>
+          <t>assets/players/real/Christopher Balraj.png</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -8321,12 +8321,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>photo-13</t>
+          <t>photo-08</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Matchday Preparation &amp; Focus</t>
+          <t>Leg-Spin Craftsmanship</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -8341,7 +8341,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>assets/players/real/Jason-Edwards.jpg</t>
+          <t>assets/players/real/Ravneet-Verma-solo.jpg</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -8353,17 +8353,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>photo-14</t>
+          <t>photo-09</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Outfield Athleticism &amp; Agility</t>
+          <t>Fast Bowling Mechanics</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -8373,7 +8373,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>assets/players/real/Jibin-Moncy.jpg</t>
+          <t>assets/players/real/Sahil-Singh.jpeg</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -8385,12 +8385,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>photo-15</t>
+          <t>photo-10</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Left-Arm Swing Trajectory</t>
+          <t>All-Round Power Hitting</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -8405,7 +8405,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>assets/players/real/Teammate-left.jpg</t>
+          <t>assets/players/real/Sakthivel shanmugasundaram.Jpg</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -8417,12 +8417,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>photo-16</t>
+          <t>photo-11</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Wicketkeeper &amp; Glovework Drills</t>
+          <t>Powerplay Strike Execution</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -8432,12 +8432,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>assets/players/real/Rajasekhara-Kalagotla.jpg</t>
+          <t>assets/players/real/Praisewin-Vincent-solo.jpg</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -8449,12 +8449,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>photo-17</t>
+          <t>photo-12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>All-Round Match Tempo</t>
+          <t>Death Overs Range Hitting</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -8464,12 +8464,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Matchday Action</t>
+          <t>Training &amp; Youth</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>assets/players/real/Fahad.JPG</t>
+          <t>assets/players/real/Viran.jpg</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -8481,30 +8481,190 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>photo-13</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Matchday Preparation &amp; Focus</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Training &amp; Youth</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>assets/players/real/Jason-Edwards.jpg</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>photo-14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Outfield Athleticism &amp; Agility</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Training &amp; Youth</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>assets/players/real/Jibin-Moncy.jpg</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>photo-15</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Left-Arm Swing Trajectory</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Matchday Action</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>assets/players/real/Teammate-left.jpg</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>photo-16</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Wicketkeeper &amp; Glovework Drills</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Training &amp; Youth</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>assets/players/real/Rajasekhara-Kalagotla.jpg</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>photo-17</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>All-Round Match Tempo</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Matchday Action</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>assets/players/real/Fahad.JPG</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>photo-18</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Franchise Management &amp; Strategy</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Behind the Scenes</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>assets/players/real/Majin-Paul-solo.jpg</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>

<commit_message>
Add official videos section, video lightbox player, and media switcher to gallery
</commit_message>
<xml_diff>
--- a/exports/Cayman_Super_Kings_Complete_Database.xlsx
+++ b/exports/Cayman_Super_Kings_Complete_Database.xlsx
@@ -7905,768 +7905,1504 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t>Image ID</t>
+          <t>Media ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr" s="1">
         <is>
-          <t>Title / Caption</t>
+          <t>Media Type</t>
         </is>
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr" s="1">
+      <c r="E1" t="inlineStr" s="1">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="1">
-        <is>
-          <t>High-Res Image Path</t>
-        </is>
-      </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
-          <t>Tags</t>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t>Media Asset Path</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t>Poster Thumbnail</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t>Caption</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>photo-00</t>
+          <t>video-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Australian Cricket Legend David Warner in Cayman</t>
+          <t>VIDEO</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Academy Batting Net Drills</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>assets/players/real/david-warner-csk-cayman.jpg</t>
+          <t>Training &amp; Youth</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t/>
+          <t>0:30</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>video/csk-match-clip-01.mp4</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>assets/videos/posters/video-01.jpg</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Junior Super King fine-tuning forward defensive technique and bat flow in the outdoor batting cages.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>photo-19</t>
+          <t>video-02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Junior Super King at the Crease</t>
+          <t>VIDEO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Bowling Machine Match Simulation</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Training &amp; Youth</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>assets/players/real/csk-youth-batting-technique.jpg</t>
-        </is>
-      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t/>
+          <t>1:21</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>video/csk-match-clip-02.mp4</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>assets/videos/posters/video-02.jpg</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Intense powerplay batting drill facing high-speed deliveries from the club bowling machine at the training facility.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>photo-20</t>
+          <t>video-03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Spirit of Cricket - Mid-Pitch Camaraderie</t>
+          <t>VIDEO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Junior Agility &amp; Crease Footwork</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Matchday Action</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>assets/players/real/csk-matchday-spirit-handshake.jpg</t>
+          <t>Training &amp; Youth</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t/>
+          <t>0:13</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>video/csk-match-clip-03.mp4</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>assets/videos/posters/video-03.jpg</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Agility marker routines designed to build quick lateral movement, balance, and quick feet at the batting crease.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>photo-21</t>
+          <t>video-04</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Taking the Field at Jimmy Powell Oval</t>
+          <t>VIDEO</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Forward Stride &amp; Precision Timing</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Matchday Action</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>assets/players/real/csk-matchday-field-stride.jpg</t>
+          <t>Training &amp; Youth</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t/>
+          <t>0:15</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>video/csk-match-clip-04.mp4</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>assets/videos/posters/video-04.jpg</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Developing head position over the ball and high elbow execution during specialized youth coaching drills.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>photo-22</t>
+          <t>video-05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Powerplay Strategy in Motion</t>
+          <t>VIDEO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Open Turf Batting Session</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Matchday Action</t>
-        </is>
-      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>assets/players/real/csk-matchday-pitch-walk.jpg</t>
+          <t>Training &amp; Youth</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t/>
+          <t>1:21</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>video/csk-match-clip-05.mp4</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>assets/videos/posters/video-05.jpg</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Full-length outdoor practice strip batting repetitions simulating real matchday bounce and trajectory.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>photo-23</t>
+          <t>video-06</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Matchday Protocol &amp; Walk-Out</t>
+          <t>VIDEO</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>Matchday Outfield Fielding Action</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Matchday Action</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>assets/players/real/csk-matchday-officials-crease.jpg</t>
-        </is>
-      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t/>
+          <t>0:25</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>video/csk-match-clip-06.mp4</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>assets/videos/posters/video-06.jpg</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings outfielders organizing defensive field placements along the boundary line at Jimmy Powell Oval.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>photo-01</t>
+          <t>video-07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Championship Squad Triumph</t>
+          <t>VIDEO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>Caribbean Rain Delay &amp; Pitch Covers</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Trophy Celebrations</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>assets/players/real/Team.jpg</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t/>
+          <t>0:41</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>video/csk-match-clip-07.mp4</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>assets/videos/posters/video-07.jpg</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>All hands on deck as ground staff and team personnel rush to protect the Jimmy Powell Oval wicket during a tropical shower.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>photo-02</t>
+          <t>video-08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Championship Matchday Action</t>
+          <t>VIDEO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>Skipper Rahul Garg Tactical Consultation</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>Matchday Action</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>assets/players/real/20250405_104447_IMG_5374.jpg</t>
-        </is>
-      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t/>
+          <t>0:15</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>video/csk-match-clip-08.mp4</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>assets/videos/posters/video-08.jpg</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Captain Rahul Garg (#38) consulting with match official at mid-off on match strategy and playing conditions.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>photo-03</t>
+          <t>photo-00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Skipper Rahul Garg Leading the Pride</t>
+          <t>PHOTO</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>Australian Cricket Legend David Warner in Cayman</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Behind the Scenes</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>assets/players/real/Rahul-Garg-Portrait.jpg</t>
-        </is>
-      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>assets/players/real/david-warner-csk-cayman.jpg</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>World Cup champion &amp; Australian cricket icon David Warner visiting Grand Cayman, connecting with Cayman Super Kings on Seven Mile Beach.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>photo-04</t>
+          <t>photo-19</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>The Founding Visionaries</t>
+          <t>PHOTO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Junior Super King at the Crease</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Behind the Scenes</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>assets/players/real/Rahul and Chris.jpg</t>
+          <t>Training &amp; Youth</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>assets/players/real/csk-youth-batting-technique.jpg</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Young Cayman cricket talent displaying textbook forward defensive technique during CSK youth academy matchday at Jimmy Powell Oval.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>photo-06</t>
+          <t>photo-20</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Wicketkeeper Reflexes</t>
+          <t>PHOTO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>Spirit of Cricket - Mid-Pitch Camaraderie</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Matchday Action</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>assets/players/real/Gokul Krishnan.jpg</t>
-        </is>
-      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>assets/players/real/csk-matchday-spirit-handshake.jpg</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Cayman Super Kings and opponent batsman sharing a handshake in the spirit of the game under the Cayman sun.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>photo-07</t>
+          <t>photo-21</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Christopher Balraj Bermuda Qualifiers</t>
+          <t>PHOTO</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Taking the Field at Jimmy Powell Oval</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>Matchday Action</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>assets/players/real/Christopher Balraj.png</t>
-        </is>
-      </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>assets/players/real/csk-matchday-field-stride.jpg</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>CSK batsman walking out alongside match officials and opponents as the afternoon session gets underway.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>photo-08</t>
+          <t>photo-22</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Leg-Spin Craftsmanship</t>
+          <t>PHOTO</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>Powerplay Strategy in Motion</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>assets/players/real/Ravneet-Verma-solo.jpg</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>assets/players/real/csk-matchday-pitch-walk.jpg</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Batsman and match officials proceeding across the turf ahead of the opening powerplay overs.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>photo-09</t>
+          <t>photo-23</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Fast Bowling Mechanics</t>
+          <t>PHOTO</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>Matchday Protocol &amp; Walk-Out</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Training &amp; Youth</t>
-        </is>
-      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>assets/players/real/Sahil-Singh.jpeg</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>assets/players/real/csk-matchday-officials-crease.jpg</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Approaching the crease at Jimmy Powell Oval for official competitive Cayman cricket fixture action.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>photo-10</t>
+          <t>photo-01</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>All-Round Power Hitting</t>
+          <t>PHOTO</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>Championship Squad Triumph</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Matchday Action</t>
-        </is>
-      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>assets/players/real/Sakthivel shanmugasundaram.Jpg</t>
+          <t>Trophy Celebrations</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>assets/players/real/Team.jpg</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>The complete Cayman Super Kings playing XI and coaching staff celebrating championship tournament qualification.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>photo-11</t>
+          <t>photo-02</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Powerplay Strike Execution</t>
+          <t>PHOTO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>Championship Matchday Action</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Matchday Action</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>assets/players/real/Praisewin-Vincent-solo.jpg</t>
-        </is>
-      </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>assets/players/real/20250405_104447_IMG_5374.jpg</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>High-stakes league competition under the Caribbean sun at Jimmy Powell Oval.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>photo-12</t>
+          <t>photo-03</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Death Overs Range Hitting</t>
+          <t>PHOTO</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>Skipper Rahul Garg Leading the Pride</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>assets/players/real/Viran.jpg</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>assets/players/real/Rahul-Garg-Portrait.jpg</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Captain Rahul Garg in official club whites ready for the 2026 CICA season campaign.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>photo-13</t>
+          <t>photo-04</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Matchday Preparation &amp; Focus</t>
+          <t>PHOTO</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>The Founding Visionaries</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>assets/players/real/Jason-Edwards.jpg</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>assets/players/real/Rahul and Chris.jpg</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Co-Founders Rahul Garg &amp; Christopher Balraj sharing strategic insights ahead of fixture season.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>photo-14</t>
+          <t>photo-06</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Outfield Athleticism &amp; Agility</t>
+          <t>PHOTO</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>Wicketkeeper Reflexes</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>assets/players/real/Jibin-Moncy.jpg</t>
+          <t>Matchday Action</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>assets/players/real/Gokul Krishnan.jpg</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Vice Captain Gokul Krishnan exhibiting lightning-quick glovework behind the wickets.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>photo-15</t>
+          <t>photo-07</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Left-Arm Swing Trajectory</t>
+          <t>PHOTO</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>Christopher Balraj Bermuda Qualifiers</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
           <t>Matchday Action</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>assets/players/real/Teammate-left.jpg</t>
-        </is>
-      </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>assets/players/real/Christopher Balraj.png</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Christopher Balraj representing the Cayman Islands national team at the Sub-Regional World Cup Qualifiers in Bermuda.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>photo-16</t>
+          <t>photo-08</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Wicketkeeper &amp; Glovework Drills</t>
+          <t>PHOTO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>Leg-Spin Craftsmanship</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Training &amp; Youth</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>assets/players/real/Rajasekhara-Kalagotla.jpg</t>
-        </is>
-      </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>assets/players/real/Ravneet-Verma-solo.jpg</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Ravneet Verma locking in variations and flight revolutions during mid-week net drills.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>photo-17</t>
+          <t>photo-09</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>All-Round Match Tempo</t>
+          <t>PHOTO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>Fast Bowling Mechanics</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Matchday Action</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>assets/players/real/Fahad.JPG</t>
+          <t>Training &amp; Youth</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>assets/players/real/Sahil-Singh.jpeg</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Strike fast bowler Sahil Singh analyzing seam alignment and front-foot release.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>photo-10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PHOTO</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>All-Round Power Hitting</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Matchday Action</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>assets/players/real/Sakthivel shanmugasundaram.Jpg</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Sakthivel Shanmugasundaram taking on the bowling attack with clean lofted drives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>photo-11</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>PHOTO</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Powerplay Strike Execution</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Matchday Action</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>assets/players/real/Praisewin-Vincent-solo.jpg</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Praisewin Vincent executing calculated aggression through the off-side during training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>photo-12</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PHOTO</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Death Overs Range Hitting</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Training &amp; Youth</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>assets/players/real/Viran.jpg</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Viran Narayana fine-tuning explosive lower-order finish execution against pace and spin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>photo-13</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PHOTO</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Matchday Preparation &amp; Focus</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Training &amp; Youth</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>assets/players/real/Jason-Edwards.jpg</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Jason Edwards completing match warmups and equipment checks before the fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>photo-14</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PHOTO</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Outfield Athleticism &amp; Agility</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Training &amp; Youth</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>assets/players/real/Jibin-Moncy.jpg</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Jibin Moncy executing high-speed boundary cut-offs and direct-hit fielding drills.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>photo-15</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PHOTO</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Left-Arm Swing Trajectory</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Matchday Action</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>assets/players/real/Teammate-left.jpg</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Muhammed Jazeem Keloth delivering swinging deliveries under match pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>photo-16</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>PHOTO</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Wicketkeeper &amp; Glovework Drills</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Training &amp; Youth</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>assets/players/real/Rajasekhara-Kalagotla.jpg</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Rajasekhara Kalagotla running through reflex gathering and stump-to-stump agility routines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>photo-17</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>PHOTO</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>All-Round Match Tempo</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Matchday Action</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>assets/players/real/Fahad.JPG</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Fahad Noushad displaying balance and strokeplay execution during match play.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>photo-18</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>PHOTO</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
         <is>
           <t>Franchise Management &amp; Strategy</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Behind the Scenes</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
         <is>
           <t>assets/players/real/Majin-Paul-solo.jpg</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Co-Founder and Team Manager Majin Paul directing logistics and tournament preparation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update gallery with truthful player names/captions, remove whistle icon, add floodlights to all page heroes, and upgrade gallery UI/UX
</commit_message>
<xml_diff>
--- a/exports/Cayman_Super_Kings_Complete_Database.xlsx
+++ b/exports/Cayman_Super_Kings_Complete_Database.xlsx
@@ -3625,7 +3625,7 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>assets/players/real/Sahil-Singh-RoyalBlue.jpg</t>
+          <t>assets/players/real/Sahil-Singh-RoyalBlue.jpg?v=20261018_short</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
@@ -7962,7 +7962,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Academy Batting Net Drills</t>
+          <t>Youth Batting Net Practice</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Junior Super King fine-tuning forward defensive technique and bat flow in the outdoor batting cages.</t>
+          <t>Video of youth batting practice in the outdoor cricket nets.</t>
         </is>
       </c>
     </row>
@@ -8009,7 +8009,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bowling Machine Match Simulation</t>
+          <t>Youth Batting Cage Session</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -8039,7 +8039,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Intense powerplay batting drill facing high-speed deliveries from the club bowling machine at the training facility.</t>
+          <t>Video of youth batting practice in the outdoor batting cage.</t>
         </is>
       </c>
     </row>
@@ -8056,7 +8056,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Junior Agility &amp; Crease Footwork</t>
+          <t>Youth Footwork &amp; Batting Drill</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -8086,7 +8086,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Agility marker routines designed to build quick lateral movement, balance, and quick feet at the batting crease.</t>
+          <t>Video of a young batter practicing footwork and batting drills on cones.</t>
         </is>
       </c>
     </row>
@@ -8103,7 +8103,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Forward Stride &amp; Precision Timing</t>
+          <t>Youth Front-Foot Batting Drill</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -8133,7 +8133,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Developing head position over the ball and high elbow execution during specialized youth coaching drills.</t>
+          <t>Video of a young batter practicing front-foot drives off cones in the nets.</t>
         </is>
       </c>
     </row>
@@ -8150,7 +8150,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Open Turf Batting Session</t>
+          <t>Outdoor Net Batting Session</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -8180,7 +8180,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Full-length outdoor practice strip batting repetitions simulating real matchday bounce and trajectory.</t>
+          <t>Video of youth batting session in the outdoor practice net.</t>
         </is>
       </c>
     </row>
@@ -8197,7 +8197,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Matchday Outfield Fielding Action</t>
+          <t>Matchday at the Boundary</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Cayman Super Kings outfielders organizing defensive field placements along the boundary line at Jimmy Powell Oval.</t>
+          <t>Video from the boundary line during a match at the cricket ground.</t>
         </is>
       </c>
     </row>
@@ -8244,7 +8244,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Caribbean Rain Delay &amp; Pitch Covers</t>
+          <t>Rain Delay &amp; Pitch Covers</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>All hands on deck as ground staff and team personnel rush to protect the Jimmy Powell Oval wicket during a tropical shower.</t>
+          <t>Video of players running off the field during rain with the pitch covered.</t>
         </is>
       </c>
     </row>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Skipper Rahul Garg Tactical Consultation</t>
+          <t>Rahul Garg &amp; Match Umpire on the Field</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -8321,7 +8321,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Captain Rahul Garg (#38) consulting with match official at mid-off on match strategy and playing conditions.</t>
+          <t>Video of Captain Rahul Garg (#38) and the match umpire on the field.</t>
         </is>
       </c>
     </row>
@@ -8338,7 +8338,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Australian Cricket Legend David Warner in Cayman</t>
+          <t>David Warner &amp; Rahul Garg</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -8368,7 +8368,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>World Cup champion &amp; Australian cricket icon David Warner visiting Grand Cayman, connecting with Cayman Super Kings on Seven Mile Beach.</t>
+          <t>Image of Australian cricketer David Warner and Cayman Super Kings Captain Rahul Garg in Grand Cayman.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Junior Super King at the Crease</t>
+          <t>Youth Match Batting</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Young Cayman cricket talent displaying textbook forward defensive technique during CSK youth academy matchday at Jimmy Powell Oval.</t>
+          <t>Image of a young batter at the crease during a youth cricket match.</t>
         </is>
       </c>
     </row>
@@ -8432,7 +8432,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Spirit of Cricket - Mid-Pitch Camaraderie</t>
+          <t>Matchday Handshake on the Pitch</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -8462,7 +8462,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Cayman Super Kings and opponent batsman sharing a handshake in the spirit of the game under the Cayman sun.</t>
+          <t>Image of players shaking hands on the pitch during a match.</t>
         </is>
       </c>
     </row>
@@ -8479,7 +8479,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Taking the Field at Jimmy Powell Oval</t>
+          <t>Players &amp; Umpire on the Field</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -8509,7 +8509,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>CSK batsman walking out alongside match officials and opponents as the afternoon session gets underway.</t>
+          <t>Image of players and the match umpire walking across the field.</t>
         </is>
       </c>
     </row>
@@ -8526,7 +8526,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Powerplay Strategy in Motion</t>
+          <t>Players &amp; Match Official on Matchday</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -8556,7 +8556,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Batsman and match officials proceeding across the turf ahead of the opening powerplay overs.</t>
+          <t>Image of players and the match official walking near the pitch.</t>
         </is>
       </c>
     </row>
@@ -8573,7 +8573,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Matchday Protocol &amp; Walk-Out</t>
+          <t>Matchday on the Field</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -8603,7 +8603,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Approaching the crease at Jimmy Powell Oval for official competitive Cayman cricket fixture action.</t>
+          <t>Image of players and the match umpire on the cricket ground.</t>
         </is>
       </c>
     </row>
@@ -8620,7 +8620,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Championship Squad Triumph</t>
+          <t>Cayman Super Kings Team Photo</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -8650,7 +8650,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>The complete Cayman Super Kings playing XI and coaching staff celebrating championship tournament qualification.</t>
+          <t>Group image of the Cayman Super Kings team in official club jerseys.</t>
         </is>
       </c>
     </row>
@@ -8667,7 +8667,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Championship Matchday Action</t>
+          <t>Wicketkeeper on the Field</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -8687,7 +8687,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>assets/players/real/20250405_104447_IMG_5374.jpg</t>
+          <t>assets/players/real/20250405_104447_IMG_5374.jpg?v=20261018_upright</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -8697,7 +8697,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>High-stakes league competition under the Caribbean sun at Jimmy Powell Oval.</t>
+          <t>Image of wicketkeeper wearing keeping gloves and catching a cricket ball on the field.</t>
         </is>
       </c>
     </row>
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Skipper Rahul Garg Leading the Pride</t>
+          <t>Rahul Garg</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -8744,7 +8744,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Captain Rahul Garg in official club whites ready for the 2026 CICA season campaign.</t>
+          <t>Image of Rahul Garg, Captain of Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -8761,7 +8761,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>The Founding Visionaries</t>
+          <t>Christopher Balraj &amp; Rahul Garg</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -8791,7 +8791,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Co-Founders Rahul Garg &amp; Christopher Balraj sharing strategic insights ahead of fixture season.</t>
+          <t>Image of Christopher Balraj and Rahul Garg in Cayman Super Kings batting gear.</t>
         </is>
       </c>
     </row>
@@ -8808,7 +8808,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Wicketkeeper Reflexes</t>
+          <t>Gokul Krishnan</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Vice Captain Gokul Krishnan exhibiting lightning-quick glovework behind the wickets.</t>
+          <t>Image of Gokul Krishnan, Vice Captain of Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -8855,7 +8855,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Christopher Balraj Bermuda Qualifiers</t>
+          <t>Christopher Balraj</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -8865,7 +8865,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Matchday Action</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -8885,7 +8885,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Christopher Balraj representing the Cayman Islands national team at the Sub-Regional World Cup Qualifiers in Bermuda.</t>
+          <t>Image of Christopher Balraj, Co-Founder of Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -8902,7 +8902,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Leg-Spin Craftsmanship</t>
+          <t>Ravneet Verma</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>Trophy Celebrations</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -8932,7 +8932,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Ravneet Verma locking in variations and flight revolutions during mid-week net drills.</t>
+          <t>Image of Ravneet Verma of Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -8949,7 +8949,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Fast Bowling Mechanics</t>
+          <t>Sahil Singh &amp; Rahul Garg</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -8959,7 +8959,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -8979,7 +8979,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Strike fast bowler Sahil Singh analyzing seam alignment and front-foot release.</t>
+          <t>Image of Sahil Singh and Rahul Garg of Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -8996,7 +8996,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>All-Round Power Hitting</t>
+          <t>Sakthivel Shanmugasundaram</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -9006,7 +9006,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Matchday Action</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -9026,7 +9026,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Sakthivel Shanmugasundaram taking on the bowling attack with clean lofted drives.</t>
+          <t>Image of Sakthivel Shanmugasundaram of Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9043,7 +9043,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Powerplay Strike Execution</t>
+          <t>Praisewin Vincent</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -9053,7 +9053,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Matchday Action</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -9073,7 +9073,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Praisewin Vincent executing calculated aggression through the off-side during training.</t>
+          <t>Image of Praisewin Vincent with teammates in the stadium stands.</t>
         </is>
       </c>
     </row>
@@ -9090,7 +9090,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Death Overs Range Hitting</t>
+          <t>Viran Narayana</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -9100,7 +9100,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -9120,7 +9120,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Viran Narayana fine-tuning explosive lower-order finish execution against pace and spin.</t>
+          <t>Image of Viran Narayana of Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9137,7 +9137,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Matchday Preparation &amp; Focus</t>
+          <t>Jason Edwards</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -9147,7 +9147,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -9167,7 +9167,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Jason Edwards completing match warmups and equipment checks before the fixture.</t>
+          <t>Image of Jason Edwards of Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9184,7 +9184,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Outfield Athleticism &amp; Agility</t>
+          <t>Jibin Moncy</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -9194,7 +9194,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Jibin Moncy executing high-speed boundary cut-offs and direct-hit fielding drills.</t>
+          <t>Image of Jibin Moncy of Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9231,7 +9231,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Left-Arm Swing Trajectory</t>
+          <t>Muhammed Jazeem Keloth</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -9241,7 +9241,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Matchday Action</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -9261,7 +9261,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Muhammed Jazeem Keloth delivering swinging deliveries under match pressure.</t>
+          <t>Image of Muhammed Jazeem Keloth of Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9278,7 +9278,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Wicketkeeper &amp; Glovework Drills</t>
+          <t>Rajasekhara Kalagotla</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -9288,7 +9288,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Training &amp; Youth</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -9308,7 +9308,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Rajasekhara Kalagotla running through reflex gathering and stump-to-stump agility routines.</t>
+          <t>Image of Rajasekhara Kalagotla of Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9325,7 +9325,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>All-Round Match Tempo</t>
+          <t>Fahad Noushad</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -9335,7 +9335,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Matchday Action</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -9355,7 +9355,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Fahad Noushad displaying balance and strokeplay execution during match play.</t>
+          <t>Image of Fahad Noushad of Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9372,7 +9372,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Franchise Management &amp; Strategy</t>
+          <t>Majin Paul</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -9402,7 +9402,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Co-Founder and Team Manager Majin Paul directing logistics and tournament preparation.</t>
+          <t>Image of Majin Paul, Co-Founder &amp; Team Manager of Cayman Super Kings.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Explicitly title person photos as 'Image of [Name]' and remove all circular icons from gallery photos
</commit_message>
<xml_diff>
--- a/exports/Cayman_Super_Kings_Complete_Database.xlsx
+++ b/exports/Cayman_Super_Kings_Complete_Database.xlsx
@@ -3625,7 +3625,7 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>assets/players/real/Sahil-Singh-RoyalBlue.jpg?v=20261018_short</t>
+          <t>assets/players/real/Sahil-Singh-RoyalBlue.jpg?v=20261018_dock_smile</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Video of youth batting practice in the outdoor cricket nets.</t>
+          <t>Youth batting practice in the outdoor cricket nets.</t>
         </is>
       </c>
     </row>
@@ -8039,7 +8039,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Video of youth batting practice in the outdoor batting cage.</t>
+          <t>Youth batting practice in the outdoor batting cage.</t>
         </is>
       </c>
     </row>
@@ -8086,7 +8086,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Video of a young batter practicing footwork and batting drills on cones.</t>
+          <t>Young batter practicing footwork and batting drills.</t>
         </is>
       </c>
     </row>
@@ -8133,7 +8133,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Video of a young batter practicing front-foot drives off cones in the nets.</t>
+          <t>Young batter practicing front-foot drives in the nets.</t>
         </is>
       </c>
     </row>
@@ -8180,7 +8180,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Video of youth batting session in the outdoor practice net.</t>
+          <t>Youth batting session in the outdoor practice net.</t>
         </is>
       </c>
     </row>
@@ -8227,7 +8227,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Video from the boundary line during a match at the cricket ground.</t>
+          <t>Matchday clip from the boundary line at the cricket ground.</t>
         </is>
       </c>
     </row>
@@ -8274,7 +8274,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Video of players running off the field during rain with the pitch covered.</t>
+          <t>Players running off the field during rain with the pitch covered.</t>
         </is>
       </c>
     </row>
@@ -8321,7 +8321,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Video of Captain Rahul Garg (#38) and the match umpire on the field.</t>
+          <t>Captain Rahul Garg (#38) and the match umpire on the field.</t>
         </is>
       </c>
     </row>
@@ -8338,7 +8338,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>David Warner &amp; Rahul Garg</t>
+          <t>Image of David Warner &amp; Rahul Garg</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -8368,7 +8368,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Image of Australian cricketer David Warner and Cayman Super Kings Captain Rahul Garg in Grand Cayman.</t>
+          <t>Australian cricketer David Warner and Cayman Super Kings Captain Rahul Garg.</t>
         </is>
       </c>
     </row>
@@ -8415,7 +8415,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Image of a young batter at the crease during a youth cricket match.</t>
+          <t>Young batter at the crease during a youth cricket match.</t>
         </is>
       </c>
     </row>
@@ -8462,7 +8462,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Image of players shaking hands on the pitch during a match.</t>
+          <t>Players shaking hands on the pitch during a match.</t>
         </is>
       </c>
     </row>
@@ -8509,7 +8509,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Image of players and the match umpire walking across the field.</t>
+          <t>Players and the match umpire walking across the field.</t>
         </is>
       </c>
     </row>
@@ -8556,7 +8556,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Image of players and the match official walking near the pitch.</t>
+          <t>Players and the match official walking near the pitch.</t>
         </is>
       </c>
     </row>
@@ -8603,7 +8603,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Image of players and the match umpire on the cricket ground.</t>
+          <t>Players and the match umpire on the cricket ground.</t>
         </is>
       </c>
     </row>
@@ -8620,7 +8620,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cayman Super Kings Team Photo</t>
+          <t>Image of Cayman Super Kings Team</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -8650,7 +8650,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Group image of the Cayman Super Kings team in official club jerseys.</t>
+          <t>Cayman Super Kings team group photo in official club jerseys.</t>
         </is>
       </c>
     </row>
@@ -8697,7 +8697,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Image of wicketkeeper wearing keeping gloves and catching a cricket ball on the field.</t>
+          <t>Wicketkeeper catching a cricket ball on the field.</t>
         </is>
       </c>
     </row>
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Rahul Garg</t>
+          <t>Image of Rahul Garg</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -8744,7 +8744,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Image of Rahul Garg, Captain of Cayman Super Kings.</t>
+          <t>Rahul Garg — Captain, Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -8761,7 +8761,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Christopher Balraj &amp; Rahul Garg</t>
+          <t>Image of Christopher Balraj &amp; Rahul Garg</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -8791,7 +8791,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Image of Christopher Balraj and Rahul Garg in Cayman Super Kings batting gear.</t>
+          <t>Christopher Balraj and Rahul Garg — Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -8808,7 +8808,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Gokul Krishnan</t>
+          <t>Image of Gokul Krishnan</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Image of Gokul Krishnan, Vice Captain of Cayman Super Kings.</t>
+          <t>Gokul Krishnan — Vice Captain, Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -8855,7 +8855,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Christopher Balraj</t>
+          <t>Image of Christopher Balraj</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -8885,7 +8885,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Image of Christopher Balraj, Co-Founder of Cayman Super Kings.</t>
+          <t>Christopher Balraj — Co-Founder, Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -8902,7 +8902,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Ravneet Verma</t>
+          <t>Image of Ravneet Verma</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -8932,7 +8932,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Image of Ravneet Verma of Cayman Super Kings.</t>
+          <t>Ravneet Verma — Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -8949,7 +8949,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Sahil Singh &amp; Rahul Garg</t>
+          <t>Image of Sahil Singh &amp; Rahul Garg</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -8979,7 +8979,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Image of Sahil Singh and Rahul Garg of Cayman Super Kings.</t>
+          <t>Sahil Singh and Rahul Garg — Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -8996,7 +8996,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Sakthivel Shanmugasundaram</t>
+          <t>Image of Sakthivel Shanmugasundaram</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -9026,7 +9026,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Image of Sakthivel Shanmugasundaram of Cayman Super Kings.</t>
+          <t>Sakthivel Shanmugasundaram — Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9043,7 +9043,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Praisewin Vincent</t>
+          <t>Image of Praisewin Vincent</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -9073,7 +9073,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Image of Praisewin Vincent with teammates in the stadium stands.</t>
+          <t>Praisewin Vincent — Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9090,7 +9090,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Viran Narayana</t>
+          <t>Image of Viran Narayana</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -9120,7 +9120,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Image of Viran Narayana of Cayman Super Kings.</t>
+          <t>Viran Narayana — Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9137,7 +9137,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Jason Edwards</t>
+          <t>Image of Jason Edwards</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -9167,7 +9167,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Image of Jason Edwards of Cayman Super Kings.</t>
+          <t>Jason Edwards — Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9184,7 +9184,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Jibin Moncy</t>
+          <t>Image of Jibin Moncy</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Image of Jibin Moncy of Cayman Super Kings.</t>
+          <t>Jibin Moncy — Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9231,7 +9231,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Muhammed Jazeem Keloth</t>
+          <t>Image of Muhammed Jazeem Keloth</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -9261,7 +9261,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Image of Muhammed Jazeem Keloth of Cayman Super Kings.</t>
+          <t>Muhammed Jazeem Keloth — Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9278,7 +9278,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Rajasekhara Kalagotla</t>
+          <t>Image of Rajasekhara Kalagotla</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -9308,7 +9308,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Image of Rajasekhara Kalagotla of Cayman Super Kings.</t>
+          <t>Rajasekhara Kalagotla — Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9325,7 +9325,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Fahad Noushad</t>
+          <t>Image of Fahad Noushad</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -9355,7 +9355,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Image of Fahad Noushad of Cayman Super Kings.</t>
+          <t>Fahad Noushad — Cayman Super Kings.</t>
         </is>
       </c>
     </row>
@@ -9372,7 +9372,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Majin Paul</t>
+          <t>Image of Majin Paul</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -9402,7 +9402,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Image of Majin Paul, Co-Founder &amp; Team Manager of Cayman Super Kings.</t>
+          <t>Majin Paul — Co-Founder &amp; Team Manager, Cayman Super Kings.</t>
         </is>
       </c>
     </row>

</xml_diff>